<commit_message>
data: 自动同步金山文档 2026-07-14 12:51
</commit_message>
<xml_diff>
--- a/2026年海外客户投诉台账.xlsx
+++ b/2026年海外客户投诉台账.xlsx
@@ -1882,6 +1882,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>1、个别检验员作业要求不清晰，作业标准不明确，存在明显的主观作业意识；</t>
     </r>
     <r>
@@ -1973,6 +1979,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>1 对标中山拉通标准修订《OQC检验作业指导书》相关要求 陈国峰 6月26日</t>
     </r>
     <r>
@@ -2251,6 +2263,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>1.生产此订单面板时，因防呆块放置在左侧，丝印商标位置在右上角，面板放反情况下，丝印位置是平整的，在丝印时存在放反后能够正常丝印的情况</t>
     </r>
     <r>
@@ -2304,6 +2322,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>1、新增临时管控要求防呆块必须放置在丝印商标位置下方（与面板脚链对齐）。——卢干要/张建林</t>
     </r>
     <r>
@@ -2580,6 +2604,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>1 拖多预装设置专属区域，并固定人员预装。物料针对拖多生产线体（W3/W7/W13）电子膨胀阀线圈预装划分区域，增加工装台，并安排固定人员预装；预装完成后在线边按照A、B、C分箱摆放，并增加明显标贴。</t>
     </r>
     <r>
@@ -2764,6 +2794,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>1.供应商端风轮做动平衡时，员工为了提高效率加平衡片后未开机，重新测试风轮平衡量，存在生产流程漏洞，导致不良流出</t>
     </r>
     <r>
@@ -2788,6 +2824,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>1、完善风轮动平衡测试操作流程规范，增加加动平衡片后重新测试动平衡量流程，同时对该产品的动平衡工序进行定人定机顶岗，便于责任追溯。</t>
     </r>
     <r>
@@ -3004,6 +3046,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>因未见实物，根据图片初步分析可能导致料带断裂的原因为</t>
     </r>
     <r>
@@ -3294,6 +3342,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>自动焊漏：弯头插配间隙，管口清洁度，枪排堵塞等造成焊接火焰波动不稳定，导致焊点未有效渗透，氦检员工检验失效导致不良品流出</t>
     </r>
     <r>
@@ -3404,6 +3458,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>每台胀管机喇叭口成型、管口高度以及长U机每台机长U管开料长度每日专项稽查通报，从加工工艺性上提升焊接稳定性</t>
     </r>
     <r>
@@ -4231,6 +4291,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>管理根因：1、针对漏贴问题：贴纸箱序列号标贴员工贴完后应自检，纸箱扫码员工应互检纸箱序列号标贴是否漏贴，实际员工自互检失效导致漏贴一张序列号标贴的不良品流出。</t>
     </r>
     <r>
@@ -4303,6 +4369,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>1、技术质量课提供补料所需纸箱序列号，生产安排申购纸箱序列号标贴，回料后立即提供给服务补发客户。——陈欣、张宏伟 7.4</t>
     </r>
     <r>
@@ -4356,6 +4428,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>【问题描述】墨西哥A客户反馈我司打包带质量差，柜内发现不少打包带已经断了的现象，详见客户提供的照片和视频，要求我司分析改善。</t>
     </r>
     <r>
@@ -4421,6 +4499,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>综合调查，墨西哥A客户反馈的打包带断裂问题是由于打包带熔接不良导致，是多层面因素共同导致的：</t>
     </r>
     <r>
@@ -4574,6 +4658,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>将从生产管控、制程规范、装柜监控多个维度落地全流程改善措施，具体安排如下：</t>
     </r>
     <r>
@@ -4702,6 +4792,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <charset val="134"/>
+      </rPr>
       <t>【问题描述】西亚H客户反馈24K和30K冷凝器破损，详见客户提供的破损照片和铭牌照片（铭牌上有对应的客户序列号）。</t>
     </r>
     <r>
@@ -6293,7 +6389,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="125">
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6561,9 +6657,6 @@
     <xf numFmtId="49" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="176" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -6588,12 +6681,6 @@
     <xf numFmtId="49" fontId="18" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="18" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="10" fontId="18" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6601,13 +6688,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="18" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6616,16 +6697,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="176" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6872,7 +6947,7 @@
 <file path=xl/woinfos.xml><?xml version="1.0" encoding="utf-8"?>
 <woInfos xmlns="https://web.wps.cn/et/2018/main" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <bookInfo cellCmpFml="4" dbFileVersion="0" changeLogVersion="0">
-    <open main="53" threadCnt="1"/>
+    <open main="58" threadCnt="1"/>
     <sheetInfos>
       <sheetInfo cellCmpFml="4" sheetStid="3">
         <open main="5" threadCnt="1"/>
@@ -7171,7 +7246,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr codeName="Sheet1">
+  <sheetPr filterMode="1" codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Y161"/>
@@ -7366,7 +7441,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" s="24" customFormat="1" ht="128.25" spans="1:25">
+    <row r="4" s="24" customFormat="1" ht="128.25" hidden="1" spans="1:25">
       <c r="A4" s="46">
         <v>2</v>
       </c>
@@ -7438,7 +7513,7 @@
       <c r="X4" s="47"/>
       <c r="Y4" s="56"/>
     </row>
-    <row r="5" s="25" customFormat="1" ht="99.75" spans="1:25">
+    <row r="5" s="25" customFormat="1" ht="99.75" hidden="1" spans="1:25">
       <c r="A5" s="46">
         <v>3</v>
       </c>
@@ -7514,7 +7589,7 @@
       </c>
       <c r="Y5" s="61"/>
     </row>
-    <row r="6" s="25" customFormat="1" ht="128.25" spans="1:25">
+    <row r="6" s="25" customFormat="1" ht="128.25" hidden="1" spans="1:25">
       <c r="A6" s="46">
         <v>4</v>
       </c>
@@ -7590,7 +7665,7 @@
       </c>
       <c r="Y6" s="61"/>
     </row>
-    <row r="7" s="25" customFormat="1" ht="285" spans="1:25">
+    <row r="7" s="25" customFormat="1" ht="285" hidden="1" spans="1:25">
       <c r="A7" s="46">
         <v>5</v>
       </c>
@@ -7664,7 +7739,7 @@
       <c r="X7" s="60"/>
       <c r="Y7" s="61"/>
     </row>
-    <row r="8" s="25" customFormat="1" ht="117.95" customHeight="1" spans="1:25">
+    <row r="8" s="25" customFormat="1" ht="117.95" hidden="1" customHeight="1" spans="1:25">
       <c r="A8" s="46">
         <v>6</v>
       </c>
@@ -7738,7 +7813,7 @@
       <c r="X8" s="60"/>
       <c r="Y8" s="61"/>
     </row>
-    <row r="9" s="25" customFormat="1" ht="128.25" spans="1:25">
+    <row r="9" s="25" customFormat="1" ht="128.25" hidden="1" spans="1:25">
       <c r="A9" s="46">
         <v>7</v>
       </c>
@@ -7814,7 +7889,7 @@
       </c>
       <c r="Y9" s="61"/>
     </row>
-    <row r="10" ht="156.75" spans="1:25">
+    <row r="10" ht="156.75" hidden="1" spans="1:25">
       <c r="A10" s="46">
         <v>8</v>
       </c>
@@ -7892,7 +7967,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="11" ht="99.75" spans="1:25">
+    <row r="11" ht="99.75" hidden="1" spans="1:25">
       <c r="A11" s="46">
         <v>9</v>
       </c>
@@ -7966,7 +8041,7 @@
       </c>
       <c r="Y11" s="67"/>
     </row>
-    <row r="12" ht="99.75" spans="1:25">
+    <row r="12" ht="99.75" hidden="1" spans="1:25">
       <c r="A12" s="46">
         <v>10</v>
       </c>
@@ -8042,7 +8117,7 @@
       </c>
       <c r="Y12" s="67"/>
     </row>
-    <row r="13" ht="142.5" spans="1:25">
+    <row r="13" ht="142.5" hidden="1" spans="1:25">
       <c r="A13" s="46">
         <v>11</v>
       </c>
@@ -8120,7 +8195,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="14" ht="114" spans="1:25">
+    <row r="14" ht="114" hidden="1" spans="1:25">
       <c r="A14" s="46">
         <v>12</v>
       </c>
@@ -8198,7 +8273,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="15" ht="128.25" spans="1:25">
+    <row r="15" ht="128.25" hidden="1" spans="1:25">
       <c r="A15" s="46">
         <v>13</v>
       </c>
@@ -8268,7 +8343,7 @@
       </c>
       <c r="Y15" s="67"/>
     </row>
-    <row r="16" ht="114" spans="1:25">
+    <row r="16" ht="114" hidden="1" spans="1:25">
       <c r="A16" s="46">
         <v>14</v>
       </c>
@@ -8346,7 +8421,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="17" ht="114" spans="1:25">
+    <row r="17" ht="114" hidden="1" spans="1:25">
       <c r="A17" s="46">
         <v>15</v>
       </c>
@@ -8420,7 +8495,7 @@
       <c r="X17" s="48"/>
       <c r="Y17" s="67"/>
     </row>
-    <row r="18" ht="150" customHeight="1" spans="1:25">
+    <row r="18" ht="150" hidden="1" customHeight="1" spans="1:25">
       <c r="A18" s="46">
         <v>16</v>
       </c>
@@ -8494,7 +8569,7 @@
       </c>
       <c r="Y18" s="67"/>
     </row>
-    <row r="19" ht="99.75" spans="1:25">
+    <row r="19" ht="99.75" hidden="1" spans="1:25">
       <c r="A19" s="46">
         <v>17</v>
       </c>
@@ -8568,7 +8643,7 @@
       </c>
       <c r="Y19" s="67"/>
     </row>
-    <row r="20" ht="199.5" spans="1:25">
+    <row r="20" ht="199.5" hidden="1" spans="1:25">
       <c r="A20" s="46">
         <v>18</v>
       </c>
@@ -8642,7 +8717,7 @@
       <c r="X20" s="48"/>
       <c r="Y20" s="67"/>
     </row>
-    <row r="21" ht="99.75" spans="1:25">
+    <row r="21" ht="99.75" hidden="1" spans="1:25">
       <c r="A21" s="46">
         <v>19</v>
       </c>
@@ -8716,7 +8791,7 @@
       <c r="X21" s="48"/>
       <c r="Y21" s="67"/>
     </row>
-    <row r="22" ht="185.25" spans="1:25">
+    <row r="22" ht="185.25" hidden="1" spans="1:25">
       <c r="A22" s="46">
         <v>20</v>
       </c>
@@ -8790,7 +8865,7 @@
       <c r="X22" s="48"/>
       <c r="Y22" s="67"/>
     </row>
-    <row r="23" ht="85.5" customHeight="1" spans="1:25">
+    <row r="23" ht="85.5" hidden="1" customHeight="1" spans="1:25">
       <c r="A23" s="46">
         <v>21</v>
       </c>
@@ -8866,7 +8941,7 @@
       </c>
       <c r="Y23" s="67"/>
     </row>
-    <row r="24" ht="156.75" spans="1:25">
+    <row r="24" ht="156.75" hidden="1" spans="1:25">
       <c r="A24" s="46">
         <v>22</v>
       </c>
@@ -8944,7 +9019,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="25" ht="99.75" spans="1:25">
+    <row r="25" ht="99.75" hidden="1" spans="1:25">
       <c r="A25" s="46">
         <v>23</v>
       </c>
@@ -9012,7 +9087,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="26" ht="297" spans="1:25">
+    <row r="26" ht="297" hidden="1" spans="1:25">
       <c r="A26" s="46">
         <v>24</v>
       </c>
@@ -9085,7 +9160,7 @@
       </c>
       <c r="X26" s="48"/>
     </row>
-    <row r="27" ht="132" spans="1:25">
+    <row r="27" ht="132" hidden="1" spans="1:25">
       <c r="A27" s="46">
         <v>25</v>
       </c>
@@ -9160,7 +9235,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" ht="148.5" spans="1:25">
+    <row r="28" ht="148.5" hidden="1" spans="1:25">
       <c r="A28" s="46">
         <v>26</v>
       </c>
@@ -9233,7 +9308,7 @@
       </c>
       <c r="X28" s="48"/>
     </row>
-    <row r="29" ht="247.5" spans="1:25">
+    <row r="29" ht="247.5" hidden="1" spans="1:25">
       <c r="A29" s="46">
         <v>27</v>
       </c>
@@ -9306,7 +9381,7 @@
       </c>
       <c r="X29" s="48"/>
     </row>
-    <row r="30" customFormat="1" ht="128.25" spans="1:25">
+    <row r="30" customFormat="1" ht="128.25" hidden="1" spans="1:25">
       <c r="A30" s="46">
         <v>28</v>
       </c>
@@ -9380,7 +9455,7 @@
       </c>
       <c r="Y30" s="67"/>
     </row>
-    <row r="31" customFormat="1" ht="128.25" spans="1:25">
+    <row r="31" customFormat="1" ht="128.25" hidden="1" spans="1:25">
       <c r="A31" s="46">
         <v>29</v>
       </c>
@@ -9450,7 +9525,7 @@
       <c r="X31" s="48"/>
       <c r="Y31" s="67"/>
     </row>
-    <row r="32" customFormat="1" ht="142.5" spans="1:25">
+    <row r="32" customFormat="1" ht="142.5" hidden="1" spans="1:25">
       <c r="A32" s="46">
         <v>30</v>
       </c>
@@ -9526,7 +9601,7 @@
       </c>
       <c r="Y32" s="67"/>
     </row>
-    <row r="33" customFormat="1" ht="114" spans="1:25">
+    <row r="33" customFormat="1" ht="114" hidden="1" spans="1:25">
       <c r="A33" s="46">
         <v>31</v>
       </c>
@@ -9590,7 +9665,7 @@
       <c r="X33" s="48"/>
       <c r="Y33" s="67"/>
     </row>
-    <row r="34" ht="114" spans="1:25">
+    <row r="34" ht="114" hidden="1" spans="1:25">
       <c r="A34" s="46">
         <v>32</v>
       </c>
@@ -9666,7 +9741,7 @@
       </c>
       <c r="Y34" s="67"/>
     </row>
-    <row r="35" ht="142.5" spans="1:25">
+    <row r="35" ht="142.5" hidden="1" spans="1:25">
       <c r="A35" s="46">
         <v>33</v>
       </c>
@@ -9742,7 +9817,7 @@
       </c>
       <c r="Y35" s="67"/>
     </row>
-    <row r="36" ht="99.75" spans="1:25">
+    <row r="36" ht="99.75" hidden="1" spans="1:25">
       <c r="A36" s="46">
         <v>34</v>
       </c>
@@ -9818,7 +9893,7 @@
       </c>
       <c r="Y36" s="67"/>
     </row>
-    <row r="37" customFormat="1" ht="142.5" spans="1:25">
+    <row r="37" customFormat="1" ht="142.5" hidden="1" spans="1:25">
       <c r="A37" s="46">
         <v>35</v>
       </c>
@@ -9896,7 +9971,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="38" ht="148.5" spans="1:25">
+    <row r="38" ht="148.5" hidden="1" spans="1:25">
       <c r="A38" s="46">
         <v>36</v>
       </c>
@@ -9972,7 +10047,7 @@
       </c>
       <c r="Y38" s="67"/>
     </row>
-    <row r="39" ht="142.5" spans="1:25">
+    <row r="39" ht="142.5" hidden="1" spans="1:25">
       <c r="A39" s="46">
         <v>37</v>
       </c>
@@ -10048,7 +10123,7 @@
       </c>
       <c r="Y39" s="67"/>
     </row>
-    <row r="40" ht="342" spans="1:25">
+    <row r="40" ht="342" hidden="1" spans="1:25">
       <c r="A40" s="46">
         <v>38</v>
       </c>
@@ -10176,7 +10251,7 @@
       <c r="X41" s="48"/>
       <c r="Y41" s="67"/>
     </row>
-    <row r="42" ht="171" spans="1:25">
+    <row r="42" ht="171" hidden="1" spans="1:25">
       <c r="A42" s="46">
         <v>40</v>
       </c>
@@ -10250,7 +10325,7 @@
       <c r="X42" s="48"/>
       <c r="Y42" s="67"/>
     </row>
-    <row r="43" ht="342" spans="1:25">
+    <row r="43" ht="342" hidden="1" spans="1:25">
       <c r="A43" s="46">
         <v>41</v>
       </c>
@@ -10324,7 +10399,7 @@
       <c r="X43" s="48"/>
       <c r="Y43" s="67"/>
     </row>
-    <row r="44" ht="153" customHeight="1" spans="1:25">
+    <row r="44" ht="153" hidden="1" customHeight="1" spans="1:25">
       <c r="A44" s="46">
         <v>42</v>
       </c>
@@ -10396,7 +10471,7 @@
       <c r="X44" s="48"/>
       <c r="Y44" s="67"/>
     </row>
-    <row r="45" ht="163.5" customHeight="1" spans="1:25">
+    <row r="45" ht="163.5" hidden="1" customHeight="1" spans="1:25">
       <c r="A45" s="46">
         <v>43</v>
       </c>
@@ -10470,7 +10545,7 @@
       <c r="X45" s="48"/>
       <c r="Y45" s="67"/>
     </row>
-    <row r="46" ht="299.25" spans="1:25">
+    <row r="46" ht="299.25" hidden="1" spans="1:25">
       <c r="A46" s="46">
         <v>44</v>
       </c>
@@ -10544,7 +10619,7 @@
       <c r="X46" s="48"/>
       <c r="Y46" s="67"/>
     </row>
-    <row r="47" ht="149.25" customHeight="1" spans="1:25">
+    <row r="47" ht="149.25" hidden="1" customHeight="1" spans="1:25">
       <c r="A47" s="46">
         <v>45</v>
       </c>
@@ -10620,7 +10695,7 @@
       </c>
       <c r="Y47" s="67"/>
     </row>
-    <row r="48" ht="149.25" customHeight="1" spans="1:25">
+    <row r="48" ht="149.25" hidden="1" customHeight="1" spans="1:25">
       <c r="A48" s="46">
         <v>46</v>
       </c>
@@ -10698,7 +10773,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="49" ht="149.25" customHeight="1" spans="1:25">
+    <row r="49" ht="149.25" hidden="1" customHeight="1" spans="1:25">
       <c r="A49" s="46">
         <v>47</v>
       </c>
@@ -10774,7 +10849,7 @@
       </c>
       <c r="Y49" s="67"/>
     </row>
-    <row r="50" ht="114" spans="1:25">
+    <row r="50" ht="114" hidden="1" spans="1:25">
       <c r="A50" s="46">
         <v>48</v>
       </c>
@@ -10850,7 +10925,7 @@
       </c>
       <c r="Y50" s="67"/>
     </row>
-    <row r="51" ht="114" spans="1:25">
+    <row r="51" ht="114" hidden="1" spans="1:25">
       <c r="A51" s="46">
         <v>49</v>
       </c>
@@ -10924,7 +10999,7 @@
       <c r="X51" s="48"/>
       <c r="Y51" s="67"/>
     </row>
-    <row r="52" ht="128.25" spans="1:25">
+    <row r="52" ht="128.25" hidden="1" spans="1:25">
       <c r="A52" s="46">
         <v>50</v>
       </c>
@@ -10998,7 +11073,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="53" ht="384.75" spans="1:25">
+    <row r="53" ht="384.75" hidden="1" spans="1:25">
       <c r="A53" s="46">
         <v>51</v>
       </c>
@@ -11072,7 +11147,7 @@
       <c r="X53" s="48"/>
       <c r="Y53" s="67"/>
     </row>
-    <row r="54" ht="136.5" customHeight="1" spans="1:25">
+    <row r="54" ht="136.5" hidden="1" customHeight="1" spans="1:25">
       <c r="A54" s="46">
         <v>52</v>
       </c>
@@ -11144,7 +11219,7 @@
       </c>
       <c r="Y54" s="67"/>
     </row>
-    <row r="55" ht="136.5" customHeight="1" spans="1:25">
+    <row r="55" ht="136.5" hidden="1" customHeight="1" spans="1:25">
       <c r="A55" s="46">
         <v>53</v>
       </c>
@@ -11218,7 +11293,7 @@
       <c r="X55" s="48"/>
       <c r="Y55" s="67"/>
     </row>
-    <row r="56" ht="85.5" spans="1:25">
+    <row r="56" ht="85.5" hidden="1" spans="1:25">
       <c r="A56" s="46">
         <v>54</v>
       </c>
@@ -11294,7 +11369,7 @@
       </c>
       <c r="Y56" s="67"/>
     </row>
-    <row r="57" ht="99.75" spans="1:25">
+    <row r="57" ht="99.75" hidden="1" spans="1:25">
       <c r="A57" s="46">
         <v>55</v>
       </c>
@@ -11370,7 +11445,7 @@
       </c>
       <c r="Y57" s="67"/>
     </row>
-    <row r="58" ht="99.75" spans="1:25">
+    <row r="58" ht="99.75" hidden="1" spans="1:25">
       <c r="A58" s="46">
         <v>56</v>
       </c>
@@ -11448,7 +11523,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="59" ht="159" customHeight="1" spans="1:25">
+    <row r="59" ht="159" hidden="1" customHeight="1" spans="1:25">
       <c r="A59" s="46">
         <v>57</v>
       </c>
@@ -11578,7 +11653,7 @@
       <c r="X60" s="48"/>
       <c r="Y60" s="67"/>
     </row>
-    <row r="61" ht="132" customHeight="1" spans="1:25">
+    <row r="61" ht="132" hidden="1" customHeight="1" spans="1:25">
       <c r="A61" s="46">
         <v>59</v>
       </c>
@@ -11625,28 +11700,28 @@
         <v>43</v>
       </c>
       <c r="Q61" s="53"/>
-      <c r="R61" s="80" t="s">
+      <c r="R61" s="68" t="s">
         <v>398</v>
       </c>
-      <c r="S61" s="81" t="s">
+      <c r="S61" s="80" t="s">
         <v>399</v>
       </c>
-      <c r="T61" s="82" t="s">
+      <c r="T61" s="81" t="s">
         <v>400</v>
       </c>
-      <c r="U61" s="82" t="s">
+      <c r="U61" s="81" t="s">
         <v>164</v>
       </c>
-      <c r="V61" s="82" t="s">
+      <c r="V61" s="81" t="s">
         <v>64</v>
       </c>
-      <c r="W61" s="82" t="s">
+      <c r="W61" s="81" t="s">
         <v>50</v>
       </c>
       <c r="X61" s="48"/>
       <c r="Y61" s="67"/>
     </row>
-    <row r="62" ht="132" spans="1:25">
+    <row r="62" ht="132" hidden="1" spans="1:25">
       <c r="A62" s="46">
         <v>60</v>
       </c>
@@ -11699,10 +11774,10 @@
       <c r="Q62" s="53" t="s">
         <v>403</v>
       </c>
-      <c r="R62" s="83" t="s">
+      <c r="R62" s="82" t="s">
         <v>404</v>
       </c>
-      <c r="S62" s="83" t="s">
+      <c r="S62" s="82" t="s">
         <v>405</v>
       </c>
       <c r="T62" s="48" t="s">
@@ -11722,7 +11797,7 @@
       </c>
       <c r="Y62" s="67"/>
     </row>
-    <row r="63" ht="132" spans="1:25">
+    <row r="63" ht="132" hidden="1" spans="1:25">
       <c r="A63" s="46">
         <v>61</v>
       </c>
@@ -11775,7 +11850,7 @@
       <c r="Q63" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="R63" s="84" t="s">
+      <c r="R63" s="83" t="s">
         <v>408</v>
       </c>
       <c r="S63" s="72" t="s">
@@ -11798,7 +11873,7 @@
       </c>
       <c r="Y63" s="67"/>
     </row>
-    <row r="64" ht="199.15" customHeight="1" spans="1:25">
+    <row r="64" ht="199.15" hidden="1" customHeight="1" spans="1:25">
       <c r="A64" s="46">
         <v>62</v>
       </c>
@@ -11854,16 +11929,16 @@
       <c r="R64" s="68" t="s">
         <v>413</v>
       </c>
-      <c r="S64" s="85" t="s">
+      <c r="S64" s="84" t="s">
         <v>414</v>
       </c>
-      <c r="T64" s="86" t="s">
+      <c r="T64" s="85" t="s">
         <v>415</v>
       </c>
       <c r="U64" s="48" t="s">
         <v>198</v>
       </c>
-      <c r="V64" s="86" t="s">
+      <c r="V64" s="85" t="s">
         <v>64</v>
       </c>
       <c r="W64" s="48" t="s">
@@ -11876,23 +11951,23 @@
         <v>416</v>
       </c>
     </row>
-    <row r="65" ht="99.75" spans="1:25">
+    <row r="65" ht="99.75" hidden="1" spans="1:25">
       <c r="A65" s="46">
         <v>63</v>
       </c>
-      <c r="B65" s="87" t="s">
+      <c r="B65" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="C65" s="87" t="s">
+      <c r="C65" s="86" t="s">
         <v>417</v>
       </c>
-      <c r="D65" s="88" t="s">
+      <c r="D65" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E65" s="89">
+      <c r="E65" s="78">
         <v>46197</v>
       </c>
-      <c r="F65" s="89">
+      <c r="F65" s="78">
         <v>46211</v>
       </c>
       <c r="G65" s="50">
@@ -11902,73 +11977,73 @@
       <c r="H65" s="78">
         <v>46204</v>
       </c>
-      <c r="I65" s="90" t="s">
+      <c r="I65" s="87" t="s">
         <v>74</v>
       </c>
-      <c r="J65" s="87" t="s">
+      <c r="J65" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="K65" s="91" t="s">
+      <c r="K65" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="L65" s="92" t="s">
+      <c r="L65" s="89" t="s">
         <v>418</v>
       </c>
-      <c r="M65" s="92" t="s">
+      <c r="M65" s="89" t="s">
         <v>419</v>
       </c>
-      <c r="N65" s="87" t="s">
+      <c r="N65" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="O65" s="87" t="s">
+      <c r="O65" s="86" t="s">
         <v>33</v>
       </c>
       <c r="P65" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q65" s="92" t="s">
+      <c r="Q65" s="89" t="s">
         <v>420</v>
       </c>
-      <c r="R65" s="93" t="s">
+      <c r="R65" s="89" t="s">
         <v>421</v>
       </c>
-      <c r="S65" s="94" t="s">
+      <c r="S65" s="90" t="s">
         <v>422</v>
       </c>
-      <c r="T65" s="95" t="s">
+      <c r="T65" s="86" t="s">
         <v>423</v>
       </c>
-      <c r="U65" s="95" t="s">
+      <c r="U65" s="86" t="s">
         <v>48</v>
       </c>
-      <c r="V65" s="95" t="s">
+      <c r="V65" s="86" t="s">
         <v>64</v>
       </c>
-      <c r="W65" s="95" t="s">
+      <c r="W65" s="86" t="s">
         <v>35</v>
       </c>
-      <c r="X65" s="95" t="s">
+      <c r="X65" s="86" t="s">
         <v>35</v>
       </c>
-      <c r="Y65" s="92"/>
-    </row>
-    <row r="66" ht="142.5" spans="1:25">
+      <c r="Y65" s="89"/>
+    </row>
+    <row r="66" ht="142.5" hidden="1" spans="1:25">
       <c r="A66" s="46">
         <v>64</v>
       </c>
-      <c r="B66" s="87" t="s">
+      <c r="B66" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="C66" s="87" t="s">
+      <c r="C66" s="86" t="s">
         <v>368</v>
       </c>
-      <c r="D66" s="88" t="s">
+      <c r="D66" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E66" s="89">
+      <c r="E66" s="78">
         <v>46198</v>
       </c>
-      <c r="F66" s="89">
+      <c r="F66" s="78">
         <v>46212</v>
       </c>
       <c r="G66" s="50">
@@ -11978,73 +12053,73 @@
       <c r="H66" s="78">
         <v>46203</v>
       </c>
-      <c r="I66" s="90" t="s">
+      <c r="I66" s="87" t="s">
         <v>110</v>
       </c>
-      <c r="J66" s="87" t="s">
+      <c r="J66" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="K66" s="91">
+      <c r="K66" s="88">
         <v>1</v>
       </c>
-      <c r="L66" s="92" t="s">
+      <c r="L66" s="89" t="s">
         <v>424</v>
       </c>
-      <c r="M66" s="92" t="s">
+      <c r="M66" s="89" t="s">
         <v>425</v>
       </c>
-      <c r="N66" s="87" t="s">
+      <c r="N66" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="O66" s="87" t="s">
+      <c r="O66" s="86" t="s">
         <v>33</v>
       </c>
       <c r="P66" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q66" s="92" t="s">
+      <c r="Q66" s="89" t="s">
         <v>425</v>
       </c>
-      <c r="R66" s="93" t="s">
+      <c r="R66" s="89" t="s">
         <v>426</v>
       </c>
-      <c r="S66" s="94" t="s">
+      <c r="S66" s="90" t="s">
         <v>427</v>
       </c>
-      <c r="T66" s="95" t="s">
+      <c r="T66" s="86" t="s">
         <v>80</v>
       </c>
-      <c r="U66" s="95" t="s">
+      <c r="U66" s="86" t="s">
         <v>48</v>
       </c>
-      <c r="V66" s="95" t="s">
+      <c r="V66" s="86" t="s">
         <v>64</v>
       </c>
-      <c r="W66" s="95" t="s">
+      <c r="W66" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="X66" s="95" t="s">
+      <c r="X66" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="Y66" s="92"/>
-    </row>
-    <row r="67" ht="128.25" spans="1:25">
+      <c r="Y66" s="89"/>
+    </row>
+    <row r="67" ht="128.25" hidden="1" spans="1:25">
       <c r="A67" s="46">
         <v>65</v>
       </c>
-      <c r="B67" s="87" t="s">
+      <c r="B67" s="86" t="s">
         <v>108</v>
       </c>
-      <c r="C67" s="87" t="s">
+      <c r="C67" s="86" t="s">
         <v>224</v>
       </c>
-      <c r="D67" s="88" t="s">
+      <c r="D67" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E67" s="89">
+      <c r="E67" s="78">
         <v>46198</v>
       </c>
-      <c r="F67" s="89">
+      <c r="F67" s="78">
         <v>46212</v>
       </c>
       <c r="G67" s="50">
@@ -12054,551 +12129,551 @@
       <c r="H67" s="78">
         <v>46211</v>
       </c>
-      <c r="I67" s="90" t="s">
+      <c r="I67" s="87" t="s">
         <v>369</v>
       </c>
-      <c r="J67" s="87" t="s">
+      <c r="J67" s="86" t="s">
         <v>40</v>
       </c>
-      <c r="K67" s="91">
+      <c r="K67" s="88">
         <v>0.004</v>
       </c>
-      <c r="L67" s="92" t="s">
+      <c r="L67" s="89" t="s">
         <v>428</v>
       </c>
-      <c r="M67" s="92" t="s">
+      <c r="M67" s="89" t="s">
         <v>429</v>
       </c>
-      <c r="N67" s="87" t="s">
+      <c r="N67" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="O67" s="87" t="s">
+      <c r="O67" s="86" t="s">
         <v>33</v>
       </c>
       <c r="P67" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q67" s="92" t="s">
+      <c r="Q67" s="89" t="s">
         <v>430</v>
       </c>
-      <c r="R67" s="93" t="s">
+      <c r="R67" s="89" t="s">
         <v>431</v>
       </c>
-      <c r="S67" s="94" t="s">
+      <c r="S67" s="90" t="s">
         <v>432</v>
       </c>
-      <c r="T67" s="95" t="s">
+      <c r="T67" s="86" t="s">
         <v>433</v>
       </c>
-      <c r="U67" s="95" t="s">
+      <c r="U67" s="86" t="s">
         <v>136</v>
       </c>
-      <c r="V67" s="87"/>
-      <c r="W67" s="87"/>
-      <c r="X67" s="87"/>
-      <c r="Y67" s="92"/>
-    </row>
-    <row r="68" ht="156.75" spans="1:25">
+      <c r="V67" s="86"/>
+      <c r="W67" s="86"/>
+      <c r="X67" s="86"/>
+      <c r="Y67" s="89"/>
+    </row>
+    <row r="68" ht="156.75" hidden="1" spans="1:25">
       <c r="A68" s="46">
         <v>66</v>
       </c>
-      <c r="B68" s="87" t="s">
+      <c r="B68" s="86" t="s">
         <v>142</v>
       </c>
-      <c r="C68" s="87" t="s">
+      <c r="C68" s="86" t="s">
         <v>152</v>
       </c>
-      <c r="D68" s="88" t="s">
+      <c r="D68" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E68" s="89">
+      <c r="E68" s="78">
         <v>46199</v>
       </c>
-      <c r="F68" s="89">
+      <c r="F68" s="78">
         <v>46213</v>
       </c>
       <c r="G68" s="50">
         <f t="shared" si="2"/>
         <v>46210</v>
       </c>
-      <c r="H68" s="96">
+      <c r="H68" s="91">
         <v>46205</v>
       </c>
-      <c r="I68" s="90" t="s">
+      <c r="I68" s="87" t="s">
         <v>74</v>
       </c>
-      <c r="J68" s="87" t="s">
+      <c r="J68" s="86" t="s">
         <v>67</v>
       </c>
-      <c r="K68" s="91">
+      <c r="K68" s="88">
         <v>1</v>
       </c>
-      <c r="L68" s="92" t="s">
+      <c r="L68" s="89" t="s">
         <v>434</v>
       </c>
-      <c r="M68" s="92" t="s">
+      <c r="M68" s="89" t="s">
         <v>435</v>
       </c>
-      <c r="N68" s="87" t="s">
+      <c r="N68" s="86" t="s">
         <v>58</v>
       </c>
-      <c r="O68" s="87" t="s">
+      <c r="O68" s="86" t="s">
         <v>59</v>
       </c>
       <c r="P68" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q68" s="97" t="s">
+      <c r="Q68" s="92" t="s">
         <v>436</v>
       </c>
-      <c r="R68" s="93" t="s">
+      <c r="R68" s="89" t="s">
         <v>437</v>
       </c>
-      <c r="S68" s="94" t="s">
+      <c r="S68" s="90" t="s">
         <v>438</v>
       </c>
-      <c r="T68" s="95" t="s">
+      <c r="T68" s="86" t="s">
         <v>96</v>
       </c>
-      <c r="U68" s="95" t="s">
+      <c r="U68" s="86" t="s">
         <v>97</v>
       </c>
-      <c r="V68" s="95" t="s">
+      <c r="V68" s="86" t="s">
         <v>64</v>
       </c>
-      <c r="W68" s="95" t="s">
+      <c r="W68" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="X68" s="95" t="s">
+      <c r="X68" s="86" t="s">
         <v>35</v>
       </c>
-      <c r="Y68" s="93" t="s">
+      <c r="Y68" s="89" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="69" ht="96" customHeight="1" spans="1:25">
+    <row r="69" ht="96" hidden="1" customHeight="1" spans="1:25">
       <c r="A69" s="46">
         <v>67</v>
       </c>
-      <c r="B69" s="87" t="s">
+      <c r="B69" s="86" t="s">
         <v>142</v>
       </c>
-      <c r="C69" s="87" t="s">
+      <c r="C69" s="86" t="s">
         <v>143</v>
       </c>
-      <c r="D69" s="88" t="s">
+      <c r="D69" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E69" s="89">
+      <c r="E69" s="78">
         <v>46204</v>
       </c>
-      <c r="F69" s="89">
+      <c r="F69" s="78">
         <v>46218</v>
       </c>
       <c r="G69" s="50">
         <f t="shared" si="2"/>
         <v>46213</v>
       </c>
-      <c r="H69" s="96">
+      <c r="H69" s="91">
         <v>46208</v>
       </c>
-      <c r="I69" s="90" t="s">
+      <c r="I69" s="87" t="s">
         <v>74</v>
       </c>
-      <c r="J69" s="87" t="s">
+      <c r="J69" s="86" t="s">
         <v>67</v>
       </c>
-      <c r="K69" s="91" t="s">
+      <c r="K69" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="L69" s="92" t="s">
+      <c r="L69" s="89" t="s">
         <v>440</v>
       </c>
-      <c r="M69" s="92" t="s">
+      <c r="M69" s="89" t="s">
         <v>441</v>
       </c>
-      <c r="N69" s="87" t="s">
+      <c r="N69" s="86" t="s">
         <v>58</v>
       </c>
-      <c r="O69" s="87" t="s">
+      <c r="O69" s="86" t="s">
         <v>59</v>
       </c>
       <c r="P69" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q69" s="92" t="s">
+      <c r="Q69" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="R69" s="93" t="s">
+      <c r="R69" s="89" t="s">
         <v>442</v>
       </c>
-      <c r="S69" s="94" t="s">
+      <c r="S69" s="90" t="s">
         <v>443</v>
       </c>
-      <c r="T69" s="95" t="s">
+      <c r="T69" s="86" t="s">
         <v>400</v>
       </c>
-      <c r="U69" s="95" t="s">
+      <c r="U69" s="86" t="s">
         <v>87</v>
       </c>
-      <c r="V69" s="95" t="s">
+      <c r="V69" s="86" t="s">
         <v>444</v>
       </c>
-      <c r="W69" s="95" t="s">
+      <c r="W69" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="X69" s="95" t="s">
+      <c r="X69" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="Y69" s="93" t="s">
+      <c r="Y69" s="89" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="70" ht="84.75" customHeight="1" spans="1:25">
+    <row r="70" ht="84.75" hidden="1" customHeight="1" spans="1:25">
       <c r="A70" s="46">
         <v>68</v>
       </c>
-      <c r="B70" s="87" t="s">
+      <c r="B70" s="86" t="s">
         <v>37</v>
       </c>
-      <c r="C70" s="87" t="s">
+      <c r="C70" s="86" t="s">
         <v>38</v>
       </c>
-      <c r="D70" s="88" t="s">
+      <c r="D70" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E70" s="89">
+      <c r="E70" s="78">
         <v>46199</v>
       </c>
-      <c r="F70" s="89">
+      <c r="F70" s="78">
         <v>46213</v>
       </c>
       <c r="G70" s="50">
         <f t="shared" si="2"/>
         <v>46210</v>
       </c>
-      <c r="H70" s="89">
+      <c r="H70" s="78">
         <v>46203</v>
       </c>
-      <c r="I70" s="88" t="s">
+      <c r="I70" s="87" t="s">
         <v>74</v>
       </c>
-      <c r="J70" s="87" t="s">
+      <c r="J70" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="K70" s="91" t="s">
+      <c r="K70" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="L70" s="92" t="s">
+      <c r="L70" s="89" t="s">
         <v>446</v>
       </c>
-      <c r="M70" s="92" t="s">
+      <c r="M70" s="89" t="s">
         <v>447</v>
       </c>
-      <c r="N70" s="87" t="s">
+      <c r="N70" s="86" t="s">
         <v>42</v>
       </c>
-      <c r="O70" s="87" t="s">
+      <c r="O70" s="86" t="s">
         <v>33</v>
       </c>
       <c r="P70" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q70" s="92"/>
-      <c r="R70" s="92" t="s">
+      <c r="Q70" s="89"/>
+      <c r="R70" s="89" t="s">
         <v>448</v>
       </c>
-      <c r="S70" s="98" t="s">
+      <c r="S70" s="90" t="s">
         <v>449</v>
       </c>
-      <c r="T70" s="87" t="s">
+      <c r="T70" s="86" t="s">
         <v>80</v>
       </c>
-      <c r="U70" s="87" t="s">
+      <c r="U70" s="86" t="s">
         <v>48</v>
       </c>
-      <c r="V70" s="87" t="s">
+      <c r="V70" s="86" t="s">
         <v>64</v>
       </c>
-      <c r="W70" s="87" t="s">
+      <c r="W70" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="X70" s="87"/>
-      <c r="Y70" s="92"/>
+      <c r="X70" s="86"/>
+      <c r="Y70" s="89"/>
     </row>
     <row r="71" ht="128.25" spans="1:25">
       <c r="A71" s="46">
         <v>69</v>
       </c>
-      <c r="B71" s="87" t="s">
+      <c r="B71" s="86" t="s">
         <v>37</v>
       </c>
-      <c r="C71" s="87" t="s">
+      <c r="C71" s="86" t="s">
         <v>450</v>
       </c>
-      <c r="D71" s="88" t="s">
+      <c r="D71" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E71" s="89">
+      <c r="E71" s="78">
         <v>46202</v>
       </c>
-      <c r="F71" s="89">
+      <c r="F71" s="78">
         <v>46216</v>
       </c>
       <c r="G71" s="50">
         <f t="shared" si="2"/>
         <v>46211</v>
       </c>
-      <c r="H71" s="99">
+      <c r="H71" s="93">
         <v>46199</v>
       </c>
-      <c r="I71" s="100" t="s">
+      <c r="I71" s="94" t="s">
         <v>159</v>
       </c>
-      <c r="J71" s="87" t="s">
+      <c r="J71" s="86" t="s">
         <v>284</v>
       </c>
-      <c r="K71" s="91" t="s">
+      <c r="K71" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="L71" s="92" t="s">
+      <c r="L71" s="89" t="s">
         <v>451</v>
       </c>
-      <c r="M71" s="92" t="s">
+      <c r="M71" s="89" t="s">
         <v>452</v>
       </c>
-      <c r="N71" s="87" t="s">
+      <c r="N71" s="86" t="s">
         <v>42</v>
       </c>
-      <c r="O71" s="87" t="s">
+      <c r="O71" s="86" t="s">
         <v>33</v>
       </c>
       <c r="P71" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="Q71" s="92" t="s">
+      <c r="Q71" s="89" t="s">
         <v>453</v>
       </c>
-      <c r="R71" s="92"/>
-      <c r="S71" s="98"/>
-      <c r="T71" s="87"/>
-      <c r="U71" s="87"/>
-      <c r="V71" s="87"/>
-      <c r="W71" s="87"/>
-      <c r="X71" s="87"/>
-      <c r="Y71" s="92" t="s">
+      <c r="R71" s="89"/>
+      <c r="S71" s="90"/>
+      <c r="T71" s="86"/>
+      <c r="U71" s="86"/>
+      <c r="V71" s="86"/>
+      <c r="W71" s="86"/>
+      <c r="X71" s="86"/>
+      <c r="Y71" s="89" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="72" ht="108" customHeight="1" spans="1:25">
+    <row r="72" ht="108" hidden="1" customHeight="1" spans="1:25">
       <c r="A72" s="46">
         <v>70</v>
       </c>
-      <c r="B72" s="87" t="s">
+      <c r="B72" s="86" t="s">
         <v>72</v>
       </c>
-      <c r="C72" s="87" t="s">
+      <c r="C72" s="86" t="s">
         <v>292</v>
       </c>
-      <c r="D72" s="88" t="s">
+      <c r="D72" s="87" t="s">
         <v>28</v>
       </c>
-      <c r="E72" s="89">
+      <c r="E72" s="78">
         <v>46206</v>
       </c>
-      <c r="F72" s="89">
+      <c r="F72" s="78">
         <v>46220</v>
       </c>
       <c r="G72" s="50">
         <f t="shared" si="2"/>
         <v>46217</v>
       </c>
-      <c r="H72" s="99">
+      <c r="H72" s="93">
         <v>46209</v>
       </c>
-      <c r="I72" s="88" t="s">
+      <c r="I72" s="87" t="s">
         <v>159</v>
       </c>
-      <c r="J72" s="87" t="s">
+      <c r="J72" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="K72" s="91" t="s">
+      <c r="K72" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="L72" s="92" t="s">
+      <c r="L72" s="89" t="s">
         <v>455</v>
       </c>
-      <c r="M72" s="92" t="s">
+      <c r="M72" s="89" t="s">
         <v>456</v>
       </c>
-      <c r="N72" s="87" t="s">
+      <c r="N72" s="86" t="s">
         <v>42</v>
       </c>
-      <c r="O72" s="87" t="s">
+      <c r="O72" s="86" t="s">
         <v>33</v>
       </c>
       <c r="P72" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q72" s="92"/>
-      <c r="R72" s="80" t="s">
+      <c r="Q72" s="89"/>
+      <c r="R72" s="68" t="s">
         <v>457</v>
       </c>
-      <c r="S72" s="81" t="s">
+      <c r="S72" s="80" t="s">
         <v>458</v>
       </c>
-      <c r="T72" s="82" t="s">
+      <c r="T72" s="81" t="s">
         <v>80</v>
       </c>
-      <c r="U72" s="82" t="s">
+      <c r="U72" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="V72" s="82" t="s">
+      <c r="V72" s="81" t="s">
         <v>64</v>
       </c>
-      <c r="W72" s="82" t="s">
+      <c r="W72" s="81" t="s">
         <v>50</v>
       </c>
-      <c r="X72" s="87"/>
-      <c r="Y72" s="92"/>
-    </row>
-    <row r="73" ht="145.5" customHeight="1" spans="1:25">
+      <c r="X72" s="86"/>
+      <c r="Y72" s="89"/>
+    </row>
+    <row r="73" ht="145.5" hidden="1" customHeight="1" spans="1:25">
       <c r="A73" s="46">
         <v>71</v>
       </c>
-      <c r="B73" s="101" t="s">
+      <c r="B73" s="85" t="s">
         <v>37</v>
       </c>
-      <c r="C73" s="82" t="s">
+      <c r="C73" s="81" t="s">
         <v>450</v>
       </c>
-      <c r="D73" s="100" t="s">
+      <c r="D73" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="E73" s="102">
+      <c r="E73" s="95">
         <v>46216</v>
       </c>
-      <c r="F73" s="102">
+      <c r="F73" s="95">
         <v>46227</v>
       </c>
-      <c r="G73" s="103">
+      <c r="G73" s="96">
         <v>46224</v>
       </c>
-      <c r="H73" s="102">
+      <c r="H73" s="95">
         <v>46217</v>
       </c>
-      <c r="I73" s="100" t="s">
+      <c r="I73" s="94" t="s">
         <v>118</v>
       </c>
-      <c r="J73" s="82" t="s">
+      <c r="J73" s="81" t="s">
         <v>284</v>
       </c>
-      <c r="K73" s="104" t="s">
+      <c r="K73" s="97" t="s">
         <v>44</v>
       </c>
-      <c r="L73" s="105" t="s">
+      <c r="L73" s="98" t="s">
         <v>459</v>
       </c>
-      <c r="M73" s="105" t="s">
+      <c r="M73" s="98" t="s">
         <v>460</v>
       </c>
-      <c r="N73" s="82" t="s">
+      <c r="N73" s="81" t="s">
         <v>42</v>
       </c>
-      <c r="O73" s="82" t="s">
+      <c r="O73" s="81" t="s">
         <v>33</v>
       </c>
       <c r="P73" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q73" s="105"/>
-      <c r="R73" s="105" t="s">
+      <c r="Q73" s="98"/>
+      <c r="R73" s="98" t="s">
         <v>461</v>
       </c>
-      <c r="S73" s="81" t="s">
+      <c r="S73" s="80" t="s">
         <v>462</v>
       </c>
-      <c r="T73" s="82" t="s">
+      <c r="T73" s="81" t="s">
         <v>80</v>
       </c>
-      <c r="U73" s="82" t="s">
+      <c r="U73" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="V73" s="82" t="s">
+      <c r="V73" s="81" t="s">
         <v>64</v>
       </c>
-      <c r="W73" s="82" t="s">
+      <c r="W73" s="81" t="s">
         <v>50</v>
       </c>
-      <c r="X73" s="82"/>
-      <c r="Y73" s="106"/>
+      <c r="X73" s="81"/>
+      <c r="Y73" s="99"/>
     </row>
     <row r="74" ht="142.5" customHeight="1" spans="1:25">
       <c r="A74" s="46">
         <v>72</v>
       </c>
-      <c r="B74" s="107" t="s">
+      <c r="B74" s="100" t="s">
         <v>72</v>
       </c>
-      <c r="C74" s="108" t="s">
+      <c r="C74" s="101" t="s">
         <v>283</v>
       </c>
-      <c r="D74" s="109" t="s">
+      <c r="D74" s="102" t="s">
         <v>28</v>
       </c>
-      <c r="E74" s="110">
+      <c r="E74" s="103">
         <v>46216</v>
       </c>
-      <c r="F74" s="110">
+      <c r="F74" s="103">
         <v>46227</v>
       </c>
-      <c r="G74" s="111">
+      <c r="G74" s="104">
         <v>46224</v>
       </c>
-      <c r="H74" s="110"/>
-      <c r="I74" s="109"/>
-      <c r="J74" s="108" t="s">
+      <c r="H74" s="103"/>
+      <c r="I74" s="102"/>
+      <c r="J74" s="101" t="s">
         <v>284</v>
       </c>
-      <c r="K74" s="112" t="s">
+      <c r="K74" s="105" t="s">
         <v>44</v>
       </c>
-      <c r="L74" s="113" t="s">
+      <c r="L74" s="106" t="s">
         <v>463</v>
       </c>
-      <c r="M74" s="113" t="s">
+      <c r="M74" s="106" t="s">
         <v>460</v>
       </c>
-      <c r="N74" s="108" t="s">
+      <c r="N74" s="101" t="s">
         <v>42</v>
       </c>
-      <c r="O74" s="108" t="s">
+      <c r="O74" s="101" t="s">
         <v>33</v>
       </c>
       <c r="P74" s="48" t="s">
         <v>291</v>
       </c>
-      <c r="Q74" s="113"/>
-      <c r="R74" s="113"/>
-      <c r="S74" s="114"/>
-      <c r="T74" s="108"/>
-      <c r="U74" s="108"/>
-      <c r="V74" s="108"/>
-      <c r="W74" s="108"/>
-      <c r="X74" s="108"/>
-      <c r="Y74" s="115"/>
-    </row>
-    <row r="75" ht="142.5" customHeight="1" spans="1:25">
+      <c r="Q74" s="106"/>
+      <c r="R74" s="106"/>
+      <c r="S74" s="107"/>
+      <c r="T74" s="101"/>
+      <c r="U74" s="101"/>
+      <c r="V74" s="101"/>
+      <c r="W74" s="101"/>
+      <c r="X74" s="101"/>
+      <c r="Y74" s="108"/>
+    </row>
+    <row r="75" ht="142.5" hidden="1" customHeight="1" spans="1:25">
       <c r="A75" s="46">
         <v>73</v>
       </c>
-      <c r="B75" s="116"/>
-      <c r="C75" s="116"/>
+      <c r="B75" s="109"/>
+      <c r="C75" s="109"/>
       <c r="D75" s="63"/>
-      <c r="E75" s="117"/>
-      <c r="F75" s="117"/>
-      <c r="G75" s="117"/>
-      <c r="H75" s="117"/>
+      <c r="E75" s="110"/>
+      <c r="F75" s="110"/>
+      <c r="G75" s="110"/>
+      <c r="H75" s="110"/>
       <c r="I75" s="63"/>
       <c r="J75" s="48"/>
       <c r="K75" s="65"/>
@@ -12617,17 +12692,17 @@
       <c r="X75" s="48"/>
       <c r="Y75" s="67"/>
     </row>
-    <row r="76" ht="141.75" customHeight="1" spans="1:25">
+    <row r="76" ht="141.75" hidden="1" customHeight="1" spans="1:25">
       <c r="A76" s="46">
         <v>74</v>
       </c>
       <c r="B76" s="48"/>
       <c r="C76" s="48"/>
       <c r="D76" s="63"/>
-      <c r="E76" s="117"/>
-      <c r="F76" s="117"/>
-      <c r="G76" s="117"/>
-      <c r="H76" s="117"/>
+      <c r="E76" s="110"/>
+      <c r="F76" s="110"/>
+      <c r="G76" s="110"/>
+      <c r="H76" s="110"/>
       <c r="I76" s="63"/>
       <c r="J76" s="48"/>
       <c r="K76" s="65"/>
@@ -12646,7 +12721,7 @@
       <c r="X76" s="48"/>
       <c r="Y76" s="67"/>
     </row>
-    <row r="77" ht="141.75" customHeight="1" spans="1:25">
+    <row r="77" ht="141.75" hidden="1" customHeight="1" spans="1:25">
       <c r="A77" s="46">
         <v>75</v>
       </c>
@@ -12675,7 +12750,7 @@
       <c r="X77" s="48"/>
       <c r="Y77" s="67"/>
     </row>
-    <row r="78" ht="16.5" spans="1:25">
+    <row r="78" ht="16.5" hidden="1" spans="1:25">
       <c r="A78" s="46">
         <v>76</v>
       </c>
@@ -12699,12 +12774,12 @@
       <c r="S78" s="53"/>
       <c r="T78" s="66"/>
       <c r="U78" s="48"/>
-      <c r="V78" s="118"/>
+      <c r="V78" s="111"/>
       <c r="W78" s="48"/>
       <c r="X78" s="48"/>
       <c r="Y78" s="67"/>
     </row>
-    <row r="79" ht="16.5" spans="1:25">
+    <row r="79" ht="16.5" hidden="1" spans="1:25">
       <c r="A79" s="46">
         <v>77</v>
       </c>
@@ -12733,7 +12808,7 @@
       <c r="X79" s="48"/>
       <c r="Y79" s="67"/>
     </row>
-    <row r="80" ht="16.5" spans="1:25">
+    <row r="80" ht="16.5" hidden="1" spans="1:25">
       <c r="A80" s="46">
         <v>78</v>
       </c>
@@ -12762,7 +12837,7 @@
       <c r="X80" s="48"/>
       <c r="Y80" s="67"/>
     </row>
-    <row r="81" ht="16.5" spans="1:25">
+    <row r="81" ht="16.5" hidden="1" spans="1:25">
       <c r="A81" s="46">
         <v>79</v>
       </c>
@@ -12791,7 +12866,7 @@
       <c r="X81" s="48"/>
       <c r="Y81" s="67"/>
     </row>
-    <row r="82" ht="16.5" spans="1:25">
+    <row r="82" ht="16.5" hidden="1" spans="1:25">
       <c r="A82" s="46">
         <v>80</v>
       </c>
@@ -12820,7 +12895,7 @@
       <c r="X82" s="48"/>
       <c r="Y82" s="67"/>
     </row>
-    <row r="83" ht="16.5" spans="1:25">
+    <row r="83" ht="16.5" hidden="1" spans="1:25">
       <c r="A83" s="46">
         <v>81</v>
       </c>
@@ -12849,7 +12924,7 @@
       <c r="X83" s="48"/>
       <c r="Y83" s="67"/>
     </row>
-    <row r="84" ht="16.5" spans="1:25">
+    <row r="84" ht="16.5" hidden="1" spans="1:25">
       <c r="A84" s="46">
         <v>82</v>
       </c>
@@ -12878,7 +12953,7 @@
       <c r="X84" s="48"/>
       <c r="Y84" s="67"/>
     </row>
-    <row r="85" ht="16.5" spans="1:25">
+    <row r="85" ht="16.5" hidden="1" spans="1:25">
       <c r="A85" s="46">
         <v>83</v>
       </c>
@@ -12907,7 +12982,7 @@
       <c r="X85" s="48"/>
       <c r="Y85" s="67"/>
     </row>
-    <row r="86" ht="16.5" spans="1:25">
+    <row r="86" ht="16.5" hidden="1" spans="1:25">
       <c r="A86" s="46">
         <v>84</v>
       </c>
@@ -12936,7 +13011,7 @@
       <c r="X86" s="48"/>
       <c r="Y86" s="67"/>
     </row>
-    <row r="87" ht="16.5" spans="1:25">
+    <row r="87" ht="16.5" hidden="1" spans="1:25">
       <c r="A87" s="46">
         <v>85</v>
       </c>
@@ -12965,7 +13040,7 @@
       <c r="X87" s="48"/>
       <c r="Y87" s="67"/>
     </row>
-    <row r="88" ht="16.5" spans="1:25">
+    <row r="88" ht="16.5" hidden="1" spans="1:25">
       <c r="A88" s="46">
         <v>86</v>
       </c>
@@ -12994,7 +13069,7 @@
       <c r="X88" s="48"/>
       <c r="Y88" s="67"/>
     </row>
-    <row r="89" ht="16.5" spans="1:25">
+    <row r="89" ht="16.5" hidden="1" spans="1:25">
       <c r="A89" s="46">
         <v>87</v>
       </c>
@@ -13023,7 +13098,7 @@
       <c r="X89" s="48"/>
       <c r="Y89" s="67"/>
     </row>
-    <row r="90" ht="16.5" spans="1:25">
+    <row r="90" ht="16.5" hidden="1" spans="1:25">
       <c r="A90" s="46">
         <v>88</v>
       </c>
@@ -13052,7 +13127,7 @@
       <c r="X90" s="48"/>
       <c r="Y90" s="67"/>
     </row>
-    <row r="91" ht="16.5" spans="1:25">
+    <row r="91" ht="16.5" hidden="1" spans="1:25">
       <c r="A91" s="46">
         <v>89</v>
       </c>
@@ -13081,7 +13156,7 @@
       <c r="X91" s="48"/>
       <c r="Y91" s="67"/>
     </row>
-    <row r="92" ht="16.5" spans="1:25">
+    <row r="92" ht="16.5" hidden="1" spans="1:25">
       <c r="A92" s="46">
         <v>90</v>
       </c>
@@ -13110,7 +13185,7 @@
       <c r="X92" s="48"/>
       <c r="Y92" s="67"/>
     </row>
-    <row r="93" ht="16.5" spans="1:25">
+    <row r="93" ht="16.5" hidden="1" spans="1:25">
       <c r="A93" s="46">
         <v>91</v>
       </c>
@@ -13139,7 +13214,7 @@
       <c r="X93" s="48"/>
       <c r="Y93" s="67"/>
     </row>
-    <row r="94" ht="16.5" spans="1:25">
+    <row r="94" ht="16.5" hidden="1" spans="1:25">
       <c r="A94" s="46">
         <v>92</v>
       </c>
@@ -13168,7 +13243,7 @@
       <c r="X94" s="48"/>
       <c r="Y94" s="67"/>
     </row>
-    <row r="95" ht="99.75" customHeight="1" spans="1:25">
+    <row r="95" ht="99.75" hidden="1" customHeight="1" spans="1:25">
       <c r="A95" s="46">
         <v>93</v>
       </c>
@@ -13197,7 +13272,7 @@
       <c r="X95" s="48"/>
       <c r="Y95" s="67"/>
     </row>
-    <row r="96" ht="146.25" customHeight="1" spans="1:25">
+    <row r="96" ht="146.25" hidden="1" customHeight="1" spans="1:25">
       <c r="A96" s="46">
         <v>94</v>
       </c>
@@ -13226,7 +13301,7 @@
       <c r="X96" s="48"/>
       <c r="Y96" s="67"/>
     </row>
-    <row r="97" ht="16.5" spans="1:25">
+    <row r="97" ht="16.5" hidden="1" spans="1:25">
       <c r="A97" s="46">
         <v>95</v>
       </c>
@@ -13255,7 +13330,7 @@
       <c r="X97" s="48"/>
       <c r="Y97" s="67"/>
     </row>
-    <row r="98" ht="122.25" customHeight="1" spans="1:25">
+    <row r="98" ht="122.25" hidden="1" customHeight="1" spans="1:25">
       <c r="A98" s="46">
         <v>96</v>
       </c>
@@ -13284,7 +13359,7 @@
       <c r="X98" s="48"/>
       <c r="Y98" s="67"/>
     </row>
-    <row r="99" ht="16.5" spans="1:25">
+    <row r="99" ht="16.5" hidden="1" spans="1:25">
       <c r="A99" s="46">
         <v>97</v>
       </c>
@@ -13313,7 +13388,7 @@
       <c r="X99" s="48"/>
       <c r="Y99" s="67"/>
     </row>
-    <row r="100" ht="16.5" spans="1:25">
+    <row r="100" ht="16.5" hidden="1" spans="1:25">
       <c r="A100" s="46">
         <v>98</v>
       </c>
@@ -13342,7 +13417,7 @@
       <c r="X100" s="48"/>
       <c r="Y100" s="67"/>
     </row>
-    <row r="101" ht="16.5" spans="1:25">
+    <row r="101" ht="16.5" hidden="1" spans="1:25">
       <c r="A101" s="46">
         <v>99</v>
       </c>
@@ -13371,7 +13446,7 @@
       <c r="X101" s="48"/>
       <c r="Y101" s="67"/>
     </row>
-    <row r="102" ht="16.5" spans="1:25">
+    <row r="102" ht="16.5" hidden="1" spans="1:25">
       <c r="A102" s="46">
         <v>100</v>
       </c>
@@ -13400,7 +13475,7 @@
       <c r="X102" s="48"/>
       <c r="Y102" s="67"/>
     </row>
-    <row r="103" ht="16.5" spans="1:25">
+    <row r="103" ht="16.5" hidden="1" spans="1:25">
       <c r="A103" s="46">
         <v>101</v>
       </c>
@@ -13429,7 +13504,7 @@
       <c r="X103" s="48"/>
       <c r="Y103" s="67"/>
     </row>
-    <row r="104" ht="16.5" spans="1:25">
+    <row r="104" ht="16.5" hidden="1" spans="1:25">
       <c r="A104" s="46">
         <v>102</v>
       </c>
@@ -13458,7 +13533,7 @@
       <c r="X104" s="48"/>
       <c r="Y104" s="67"/>
     </row>
-    <row r="105" ht="16.5" spans="1:25">
+    <row r="105" ht="16.5" hidden="1" spans="1:25">
       <c r="A105" s="46">
         <v>103</v>
       </c>
@@ -13487,7 +13562,7 @@
       <c r="X105" s="48"/>
       <c r="Y105" s="67"/>
     </row>
-    <row r="106" ht="16.5" spans="1:25">
+    <row r="106" ht="16.5" hidden="1" spans="1:25">
       <c r="A106" s="46">
         <v>104</v>
       </c>
@@ -13516,12 +13591,12 @@
       <c r="X106" s="48"/>
       <c r="Y106" s="67"/>
     </row>
-    <row r="107" ht="16.5" spans="1:25">
+    <row r="107" ht="16.5" hidden="1" spans="1:25">
       <c r="A107" s="46">
         <v>105</v>
       </c>
       <c r="B107" s="48"/>
-      <c r="C107" s="119"/>
+      <c r="C107" s="112"/>
       <c r="D107" s="63"/>
       <c r="E107" s="69"/>
       <c r="F107" s="69"/>
@@ -13545,7 +13620,7 @@
       <c r="X107" s="48"/>
       <c r="Y107" s="67"/>
     </row>
-    <row r="108" ht="16.5" spans="1:25">
+    <row r="108" ht="16.5" hidden="1" spans="1:25">
       <c r="A108" s="46">
         <v>106</v>
       </c>
@@ -13574,7 +13649,7 @@
       <c r="X108" s="48"/>
       <c r="Y108" s="67"/>
     </row>
-    <row r="109" ht="16.5" spans="1:25">
+    <row r="109" ht="16.5" hidden="1" spans="1:25">
       <c r="A109" s="46">
         <v>107</v>
       </c>
@@ -13603,7 +13678,7 @@
       <c r="X109" s="48"/>
       <c r="Y109" s="67"/>
     </row>
-    <row r="110" ht="14.25" spans="1:25">
+    <row r="110" ht="14.25" hidden="1" spans="1:25">
       <c r="A110" s="46">
         <v>108</v>
       </c>
@@ -13632,7 +13707,7 @@
       <c r="X110" s="48"/>
       <c r="Y110" s="67"/>
     </row>
-    <row r="111" ht="16.5" spans="1:25">
+    <row r="111" ht="16.5" hidden="1" spans="1:25">
       <c r="A111" s="46">
         <v>109</v>
       </c>
@@ -13654,14 +13729,14 @@
       <c r="Q111" s="53"/>
       <c r="R111" s="53"/>
       <c r="S111" s="66"/>
-      <c r="T111" s="120"/>
+      <c r="T111" s="113"/>
       <c r="U111" s="48"/>
       <c r="V111" s="48"/>
       <c r="W111" s="48"/>
       <c r="X111" s="48"/>
       <c r="Y111" s="67"/>
     </row>
-    <row r="112" ht="16.5" spans="1:25">
+    <row r="112" ht="16.5" hidden="1" spans="1:25">
       <c r="A112" s="46">
         <v>110</v>
       </c>
@@ -13683,14 +13758,14 @@
       <c r="Q112" s="53"/>
       <c r="R112" s="53"/>
       <c r="S112" s="66"/>
-      <c r="T112" s="120"/>
+      <c r="T112" s="113"/>
       <c r="U112" s="48"/>
       <c r="V112" s="48"/>
       <c r="W112" s="48"/>
       <c r="X112" s="48"/>
       <c r="Y112" s="67"/>
     </row>
-    <row r="113" ht="16.5" spans="1:25">
+    <row r="113" ht="16.5" hidden="1" spans="1:25">
       <c r="A113" s="46">
         <v>111</v>
       </c>
@@ -13719,7 +13794,7 @@
       <c r="X113" s="48"/>
       <c r="Y113" s="67"/>
     </row>
-    <row r="114" ht="16.5" spans="1:25">
+    <row r="114" ht="16.5" hidden="1" spans="1:25">
       <c r="A114" s="46">
         <v>112</v>
       </c>
@@ -13741,14 +13816,14 @@
       <c r="Q114" s="53"/>
       <c r="R114" s="53"/>
       <c r="S114" s="66"/>
-      <c r="T114" s="120"/>
+      <c r="T114" s="113"/>
       <c r="U114" s="48"/>
       <c r="V114" s="48"/>
       <c r="W114" s="48"/>
       <c r="X114" s="48"/>
       <c r="Y114" s="67"/>
     </row>
-    <row r="115" ht="16.5" spans="1:25">
+    <row r="115" ht="16.5" hidden="1" spans="1:25">
       <c r="A115" s="46">
         <v>113</v>
       </c>
@@ -13776,7 +13851,7 @@
       <c r="W115" s="48"/>
       <c r="X115" s="48"/>
     </row>
-    <row r="116" ht="16.5" spans="1:25">
+    <row r="116" ht="16.5" hidden="1" spans="1:25">
       <c r="A116" s="46">
         <v>114</v>
       </c>
@@ -13798,13 +13873,13 @@
       <c r="Q116" s="53"/>
       <c r="R116" s="53"/>
       <c r="S116" s="66"/>
-      <c r="T116" s="120"/>
+      <c r="T116" s="113"/>
       <c r="U116" s="48"/>
       <c r="V116" s="48"/>
       <c r="W116" s="48"/>
       <c r="X116" s="48"/>
     </row>
-    <row r="117" customHeight="1" spans="1:25">
+    <row r="117" hidden="1" customHeight="1" spans="1:25">
       <c r="A117" s="46">
         <v>115</v>
       </c>
@@ -13832,7 +13907,7 @@
       <c r="W117" s="48"/>
       <c r="X117" s="48"/>
     </row>
-    <row r="118" customHeight="1" spans="1:25">
+    <row r="118" hidden="1" customHeight="1" spans="1:25">
       <c r="A118" s="46">
         <v>116</v>
       </c>
@@ -13860,35 +13935,35 @@
       <c r="W118" s="48"/>
       <c r="X118" s="48"/>
     </row>
-    <row r="119" customHeight="1" spans="1:25">
+    <row r="119" hidden="1" customHeight="1" spans="1:25">
       <c r="A119" s="46">
         <v>117</v>
       </c>
-      <c r="B119" s="121"/>
-      <c r="C119" s="121"/>
-      <c r="D119" s="122"/>
-      <c r="E119" s="123"/>
-      <c r="F119" s="123"/>
-      <c r="G119" s="123"/>
-      <c r="H119" s="123"/>
-      <c r="I119" s="122"/>
-      <c r="J119" s="121"/>
-      <c r="K119" s="124"/>
-      <c r="L119" s="125"/>
-      <c r="M119" s="125"/>
-      <c r="N119" s="121"/>
-      <c r="O119" s="121"/>
-      <c r="P119" s="121"/>
-      <c r="Q119" s="125"/>
-      <c r="R119" s="125"/>
-      <c r="S119" s="126"/>
-      <c r="T119" s="121"/>
-      <c r="U119" s="121"/>
-      <c r="V119" s="121"/>
-      <c r="W119" s="121"/>
-      <c r="X119" s="121"/>
-    </row>
-    <row r="120" ht="135" customHeight="1" spans="1:25">
+      <c r="B119" s="114"/>
+      <c r="C119" s="114"/>
+      <c r="D119" s="115"/>
+      <c r="E119" s="116"/>
+      <c r="F119" s="116"/>
+      <c r="G119" s="116"/>
+      <c r="H119" s="116"/>
+      <c r="I119" s="115"/>
+      <c r="J119" s="114"/>
+      <c r="K119" s="117"/>
+      <c r="L119" s="118"/>
+      <c r="M119" s="118"/>
+      <c r="N119" s="114"/>
+      <c r="O119" s="114"/>
+      <c r="P119" s="114"/>
+      <c r="Q119" s="118"/>
+      <c r="R119" s="118"/>
+      <c r="S119" s="119"/>
+      <c r="T119" s="114"/>
+      <c r="U119" s="114"/>
+      <c r="V119" s="114"/>
+      <c r="W119" s="114"/>
+      <c r="X119" s="114"/>
+    </row>
+    <row r="120" ht="135" hidden="1" customHeight="1" spans="1:25">
       <c r="A120" s="46">
         <v>118</v>
       </c>
@@ -13917,7 +13992,7 @@
       <c r="X120" s="48"/>
       <c r="Y120" s="67"/>
     </row>
-    <row r="121" ht="108" customHeight="1" spans="1:25">
+    <row r="121" ht="108" hidden="1" customHeight="1" spans="1:25">
       <c r="A121" s="46">
         <v>119</v>
       </c>
@@ -13941,26 +14016,26 @@
       <c r="S121" s="66"/>
       <c r="T121" s="48"/>
       <c r="U121" s="48"/>
-      <c r="V121" s="121"/>
-      <c r="W121" s="121"/>
+      <c r="V121" s="114"/>
+      <c r="W121" s="114"/>
       <c r="X121" s="48"/>
       <c r="Y121" s="67"/>
     </row>
-    <row r="122" ht="187.5" customHeight="1" spans="1:25">
+    <row r="122" ht="187.5" hidden="1" customHeight="1" spans="1:25">
       <c r="A122" s="46">
         <v>120</v>
       </c>
       <c r="B122" s="48"/>
       <c r="C122" s="48"/>
       <c r="D122" s="63"/>
-      <c r="E122" s="127"/>
-      <c r="F122" s="127"/>
-      <c r="G122" s="127"/>
-      <c r="H122" s="127"/>
+      <c r="E122" s="120"/>
+      <c r="F122" s="120"/>
+      <c r="G122" s="120"/>
+      <c r="H122" s="120"/>
       <c r="I122" s="63"/>
       <c r="J122" s="48"/>
       <c r="K122" s="65"/>
-      <c r="L122" s="128"/>
+      <c r="L122" s="121"/>
       <c r="M122" s="53"/>
       <c r="N122" s="48"/>
       <c r="O122" s="48"/>
@@ -13975,17 +14050,17 @@
       <c r="X122" s="48"/>
       <c r="Y122" s="53"/>
     </row>
-    <row r="123" customHeight="1" spans="1:25">
+    <row r="123" hidden="1" customHeight="1" spans="1:25">
       <c r="A123" s="46">
         <v>121</v>
       </c>
       <c r="B123" s="48"/>
       <c r="C123" s="48"/>
       <c r="D123" s="63"/>
-      <c r="E123" s="127"/>
-      <c r="F123" s="127"/>
-      <c r="G123" s="127"/>
-      <c r="H123" s="127"/>
+      <c r="E123" s="120"/>
+      <c r="F123" s="120"/>
+      <c r="G123" s="120"/>
+      <c r="H123" s="120"/>
       <c r="I123" s="63"/>
       <c r="J123" s="48"/>
       <c r="K123" s="65"/>
@@ -14004,17 +14079,17 @@
       <c r="X123" s="48"/>
       <c r="Y123" s="67"/>
     </row>
-    <row r="124" ht="141.6" customHeight="1" spans="1:25">
+    <row r="124" ht="141.6" hidden="1" customHeight="1" spans="1:25">
       <c r="A124" s="46">
         <v>122</v>
       </c>
       <c r="B124" s="48"/>
       <c r="C124" s="48"/>
       <c r="D124" s="63"/>
-      <c r="E124" s="127"/>
-      <c r="F124" s="127"/>
-      <c r="G124" s="127"/>
-      <c r="H124" s="127"/>
+      <c r="E124" s="120"/>
+      <c r="F124" s="120"/>
+      <c r="G124" s="120"/>
+      <c r="H124" s="120"/>
       <c r="I124" s="63"/>
       <c r="J124" s="48"/>
       <c r="K124" s="65"/>
@@ -14033,17 +14108,17 @@
       <c r="X124" s="48"/>
       <c r="Y124" s="67"/>
     </row>
-    <row r="125" ht="16.5" spans="1:25">
+    <row r="125" ht="16.5" hidden="1" spans="1:25">
       <c r="A125" s="46">
         <v>123</v>
       </c>
       <c r="B125" s="48"/>
       <c r="C125" s="48"/>
       <c r="D125" s="63"/>
-      <c r="E125" s="127"/>
-      <c r="F125" s="127"/>
-      <c r="G125" s="127"/>
-      <c r="H125" s="127"/>
+      <c r="E125" s="120"/>
+      <c r="F125" s="120"/>
+      <c r="G125" s="120"/>
+      <c r="H125" s="120"/>
       <c r="I125" s="63"/>
       <c r="J125" s="48"/>
       <c r="K125" s="65"/>
@@ -14062,17 +14137,17 @@
       <c r="X125" s="48"/>
       <c r="Y125" s="67"/>
     </row>
-    <row r="126" ht="16.5" spans="1:25">
+    <row r="126" ht="16.5" hidden="1" spans="1:25">
       <c r="A126" s="46">
         <v>124</v>
       </c>
       <c r="B126" s="48"/>
       <c r="C126" s="48"/>
       <c r="D126" s="63"/>
-      <c r="E126" s="127"/>
-      <c r="F126" s="127"/>
-      <c r="G126" s="127"/>
-      <c r="H126" s="127"/>
+      <c r="E126" s="120"/>
+      <c r="F126" s="120"/>
+      <c r="G126" s="120"/>
+      <c r="H126" s="120"/>
       <c r="I126" s="63"/>
       <c r="J126" s="48"/>
       <c r="K126" s="65"/>
@@ -14091,17 +14166,17 @@
       <c r="X126" s="48"/>
       <c r="Y126" s="67"/>
     </row>
-    <row r="127" ht="316.15" customHeight="1" spans="1:25">
+    <row r="127" ht="316.15" hidden="1" customHeight="1" spans="1:25">
       <c r="A127" s="46">
         <v>125</v>
       </c>
       <c r="B127" s="48"/>
       <c r="C127" s="48"/>
       <c r="D127" s="63"/>
-      <c r="E127" s="127"/>
-      <c r="F127" s="127"/>
-      <c r="G127" s="127"/>
-      <c r="H127" s="127"/>
+      <c r="E127" s="120"/>
+      <c r="F127" s="120"/>
+      <c r="G127" s="120"/>
+      <c r="H127" s="120"/>
       <c r="I127" s="63"/>
       <c r="J127" s="48"/>
       <c r="K127" s="65"/>
@@ -14120,7 +14195,7 @@
       <c r="X127" s="48"/>
       <c r="Y127" s="67"/>
     </row>
-    <row r="128" ht="165.75" customHeight="1" spans="1:25">
+    <row r="128" ht="165.75" hidden="1" customHeight="1" spans="1:25">
       <c r="A128" s="46">
         <v>126</v>
       </c>
@@ -14140,8 +14215,8 @@
       <c r="O128" s="48"/>
       <c r="P128" s="48"/>
       <c r="Q128" s="53"/>
-      <c r="R128" s="120"/>
-      <c r="S128" s="120"/>
+      <c r="R128" s="113"/>
+      <c r="S128" s="113"/>
       <c r="T128" s="48"/>
       <c r="U128" s="48"/>
       <c r="V128" s="48"/>
@@ -14149,7 +14224,7 @@
       <c r="X128" s="48"/>
       <c r="Y128" s="67"/>
     </row>
-    <row r="129" ht="16.5" spans="1:25">
+    <row r="129" ht="16.5" hidden="1" spans="1:25">
       <c r="A129" s="46">
         <v>127</v>
       </c>
@@ -14169,8 +14244,8 @@
       <c r="O129" s="48"/>
       <c r="P129" s="48"/>
       <c r="Q129" s="53"/>
-      <c r="R129" s="129"/>
-      <c r="S129" s="130"/>
+      <c r="R129" s="122"/>
+      <c r="S129" s="123"/>
       <c r="T129" s="48"/>
       <c r="U129" s="48"/>
       <c r="V129" s="48"/>
@@ -14178,7 +14253,7 @@
       <c r="X129" s="48"/>
       <c r="Y129" s="67"/>
     </row>
-    <row r="130" ht="16.5" spans="1:25">
+    <row r="130" ht="16.5" hidden="1" spans="1:25">
       <c r="A130" s="46">
         <v>128</v>
       </c>
@@ -14207,7 +14282,7 @@
       <c r="X130" s="48"/>
       <c r="Y130" s="67"/>
     </row>
-    <row r="131" ht="16.5" spans="1:25">
+    <row r="131" ht="16.5" hidden="1" spans="1:25">
       <c r="A131" s="46">
         <v>129</v>
       </c>
@@ -14236,7 +14311,7 @@
       <c r="X131" s="48"/>
       <c r="Y131" s="67"/>
     </row>
-    <row r="132" ht="16.5" spans="1:25">
+    <row r="132" ht="16.5" hidden="1" spans="1:25">
       <c r="A132" s="46">
         <v>130</v>
       </c>
@@ -14265,7 +14340,7 @@
       <c r="X132" s="48"/>
       <c r="Y132" s="67"/>
     </row>
-    <row r="133" ht="181.5" customHeight="1" spans="1:25">
+    <row r="133" ht="181.5" hidden="1" customHeight="1" spans="1:25">
       <c r="A133" s="46">
         <v>131</v>
       </c>
@@ -14294,7 +14369,7 @@
       <c r="X133" s="48"/>
       <c r="Y133" s="67"/>
     </row>
-    <row r="134" ht="150.75" customHeight="1" spans="1:25">
+    <row r="134" ht="150.75" hidden="1" customHeight="1" spans="1:25">
       <c r="A134" s="46">
         <v>132</v>
       </c>
@@ -14323,17 +14398,17 @@
       <c r="X134" s="48"/>
       <c r="Y134" s="67"/>
     </row>
-    <row r="135" ht="108" customHeight="1" spans="1:25">
+    <row r="135" ht="108" hidden="1" customHeight="1" spans="1:25">
       <c r="A135" s="46">
         <v>133</v>
       </c>
       <c r="B135" s="48"/>
       <c r="C135" s="48"/>
       <c r="D135" s="63"/>
-      <c r="E135" s="127"/>
-      <c r="F135" s="127"/>
-      <c r="G135" s="127"/>
-      <c r="H135" s="127"/>
+      <c r="E135" s="120"/>
+      <c r="F135" s="120"/>
+      <c r="G135" s="120"/>
+      <c r="H135" s="120"/>
       <c r="I135" s="63"/>
       <c r="J135" s="48"/>
       <c r="K135" s="65"/>
@@ -14352,17 +14427,17 @@
       <c r="X135" s="48"/>
       <c r="Y135" s="67"/>
     </row>
-    <row r="136" ht="16.5" spans="1:25">
+    <row r="136" ht="16.5" hidden="1" spans="1:25">
       <c r="A136" s="46">
         <v>134</v>
       </c>
       <c r="B136" s="48"/>
       <c r="C136" s="48"/>
       <c r="D136" s="63"/>
-      <c r="E136" s="127"/>
-      <c r="F136" s="127"/>
-      <c r="G136" s="127"/>
-      <c r="H136" s="127"/>
+      <c r="E136" s="120"/>
+      <c r="F136" s="120"/>
+      <c r="G136" s="120"/>
+      <c r="H136" s="120"/>
       <c r="I136" s="63"/>
       <c r="J136" s="48"/>
       <c r="K136" s="65"/>
@@ -14381,17 +14456,17 @@
       <c r="X136" s="48"/>
       <c r="Y136" s="67"/>
     </row>
-    <row r="137" ht="16.5" spans="1:25">
+    <row r="137" ht="16.5" hidden="1" spans="1:25">
       <c r="A137" s="46">
         <v>135</v>
       </c>
       <c r="B137" s="48"/>
       <c r="C137" s="48"/>
       <c r="D137" s="63"/>
-      <c r="E137" s="127"/>
-      <c r="F137" s="127"/>
-      <c r="G137" s="127"/>
-      <c r="H137" s="127"/>
+      <c r="E137" s="120"/>
+      <c r="F137" s="120"/>
+      <c r="G137" s="120"/>
+      <c r="H137" s="120"/>
       <c r="I137" s="63"/>
       <c r="J137" s="48"/>
       <c r="K137" s="65"/>
@@ -14410,7 +14485,7 @@
       <c r="X137" s="48"/>
       <c r="Y137" s="67"/>
     </row>
-    <row r="138" ht="16.5" spans="1:25">
+    <row r="138" ht="16.5" hidden="1" spans="1:25">
       <c r="A138" s="46">
         <v>136</v>
       </c>
@@ -14420,7 +14495,7 @@
       <c r="E138" s="69"/>
       <c r="F138" s="69"/>
       <c r="G138" s="69"/>
-      <c r="H138" s="127"/>
+      <c r="H138" s="120"/>
       <c r="I138" s="63"/>
       <c r="J138" s="48"/>
       <c r="K138" s="65"/>
@@ -14439,17 +14514,17 @@
       <c r="X138" s="48"/>
       <c r="Y138" s="67"/>
     </row>
-    <row r="139" ht="16.5" spans="1:25">
+    <row r="139" ht="16.5" hidden="1" spans="1:25">
       <c r="A139" s="46">
         <v>137</v>
       </c>
       <c r="B139" s="48"/>
       <c r="C139" s="48"/>
       <c r="D139" s="63"/>
-      <c r="E139" s="127"/>
-      <c r="F139" s="127"/>
-      <c r="G139" s="127"/>
-      <c r="H139" s="127"/>
+      <c r="E139" s="120"/>
+      <c r="F139" s="120"/>
+      <c r="G139" s="120"/>
+      <c r="H139" s="120"/>
       <c r="I139" s="63"/>
       <c r="J139" s="48"/>
       <c r="K139" s="65"/>
@@ -14468,17 +14543,17 @@
       <c r="X139" s="48"/>
       <c r="Y139" s="67"/>
     </row>
-    <row r="140" ht="16.5" spans="1:25">
+    <row r="140" ht="16.5" hidden="1" spans="1:25">
       <c r="A140" s="46">
         <v>138</v>
       </c>
       <c r="B140" s="48"/>
       <c r="C140" s="48"/>
       <c r="D140" s="63"/>
-      <c r="E140" s="131"/>
-      <c r="F140" s="127"/>
-      <c r="G140" s="127"/>
-      <c r="H140" s="127"/>
+      <c r="E140" s="124"/>
+      <c r="F140" s="120"/>
+      <c r="G140" s="120"/>
+      <c r="H140" s="120"/>
       <c r="I140" s="63"/>
       <c r="J140" s="48"/>
       <c r="K140" s="65"/>
@@ -14497,17 +14572,17 @@
       <c r="X140" s="48"/>
       <c r="Y140" s="67"/>
     </row>
-    <row r="141" ht="16.5" spans="1:25">
+    <row r="141" ht="16.5" hidden="1" spans="1:25">
       <c r="A141" s="46">
         <v>139</v>
       </c>
       <c r="B141" s="48"/>
       <c r="C141" s="48"/>
       <c r="D141" s="63"/>
-      <c r="E141" s="127"/>
-      <c r="F141" s="127"/>
-      <c r="G141" s="127"/>
-      <c r="H141" s="127"/>
+      <c r="E141" s="120"/>
+      <c r="F141" s="120"/>
+      <c r="G141" s="120"/>
+      <c r="H141" s="120"/>
       <c r="I141" s="63"/>
       <c r="J141" s="48"/>
       <c r="K141" s="65"/>
@@ -14526,17 +14601,17 @@
       <c r="X141" s="48"/>
       <c r="Y141" s="67"/>
     </row>
-    <row r="142" ht="16.5" spans="1:25">
+    <row r="142" ht="16.5" hidden="1" spans="1:25">
       <c r="A142" s="46">
         <v>140</v>
       </c>
       <c r="B142" s="48"/>
       <c r="C142" s="48"/>
       <c r="D142" s="63"/>
-      <c r="E142" s="127"/>
-      <c r="F142" s="127"/>
-      <c r="G142" s="127"/>
-      <c r="H142" s="127"/>
+      <c r="E142" s="120"/>
+      <c r="F142" s="120"/>
+      <c r="G142" s="120"/>
+      <c r="H142" s="120"/>
       <c r="I142" s="63"/>
       <c r="J142" s="48"/>
       <c r="K142" s="65"/>
@@ -14555,17 +14630,17 @@
       <c r="X142" s="48"/>
       <c r="Y142" s="67"/>
     </row>
-    <row r="143" ht="16.5" spans="1:25">
+    <row r="143" ht="16.5" hidden="1" spans="1:25">
       <c r="A143" s="46">
         <v>141</v>
       </c>
       <c r="B143" s="48"/>
       <c r="C143" s="48"/>
       <c r="D143" s="63"/>
-      <c r="E143" s="127"/>
-      <c r="F143" s="127"/>
-      <c r="G143" s="127"/>
-      <c r="H143" s="127"/>
+      <c r="E143" s="120"/>
+      <c r="F143" s="120"/>
+      <c r="G143" s="120"/>
+      <c r="H143" s="120"/>
       <c r="I143" s="63"/>
       <c r="J143" s="48"/>
       <c r="K143" s="65"/>
@@ -14584,14 +14659,14 @@
       <c r="X143" s="48"/>
       <c r="Y143" s="67"/>
     </row>
-    <row r="144" ht="16.5" spans="1:25">
+    <row r="144" ht="16.5" hidden="1" spans="1:25">
       <c r="A144" s="46">
         <v>142</v>
       </c>
       <c r="B144" s="48"/>
       <c r="C144" s="48"/>
       <c r="D144" s="63"/>
-      <c r="E144" s="131"/>
+      <c r="E144" s="124"/>
       <c r="F144" s="50"/>
       <c r="G144" s="50"/>
       <c r="H144" s="50"/>
@@ -14605,7 +14680,7 @@
       <c r="P144" s="48"/>
       <c r="Q144" s="53"/>
       <c r="R144" s="53"/>
-      <c r="S144" s="130"/>
+      <c r="S144" s="123"/>
       <c r="T144" s="48"/>
       <c r="U144" s="48"/>
       <c r="V144" s="48"/>
@@ -14613,7 +14688,7 @@
       <c r="X144" s="48"/>
       <c r="Y144" s="67"/>
     </row>
-    <row r="145" ht="16.5" spans="1:25">
+    <row r="145" ht="16.5" hidden="1" spans="1:25">
       <c r="A145" s="46">
         <v>143</v>
       </c>
@@ -14642,7 +14717,7 @@
       <c r="X145" s="48"/>
       <c r="Y145" s="67"/>
     </row>
-    <row r="146" ht="16.5" spans="1:25">
+    <row r="146" ht="16.5" hidden="1" spans="1:25">
       <c r="A146" s="46">
         <v>144</v>
       </c>
@@ -14671,7 +14746,7 @@
       <c r="X146" s="48"/>
       <c r="Y146" s="67"/>
     </row>
-    <row r="147" ht="16.5" spans="1:25">
+    <row r="147" ht="16.5" hidden="1" spans="1:25">
       <c r="A147" s="46">
         <v>145</v>
       </c>
@@ -14681,7 +14756,7 @@
       <c r="E147" s="64"/>
       <c r="F147" s="64"/>
       <c r="G147" s="64"/>
-      <c r="H147" s="127"/>
+      <c r="H147" s="120"/>
       <c r="I147" s="63"/>
       <c r="J147" s="48"/>
       <c r="K147" s="65"/>
@@ -14700,7 +14775,7 @@
       <c r="X147" s="48"/>
       <c r="Y147" s="67"/>
     </row>
-    <row r="148" ht="16.5" spans="1:25">
+    <row r="148" ht="16.5" hidden="1" spans="1:25">
       <c r="A148" s="46">
         <v>146</v>
       </c>
@@ -14710,7 +14785,7 @@
       <c r="E148" s="64"/>
       <c r="F148" s="64"/>
       <c r="G148" s="64"/>
-      <c r="H148" s="127"/>
+      <c r="H148" s="120"/>
       <c r="I148" s="63"/>
       <c r="J148" s="48"/>
       <c r="K148" s="65"/>
@@ -14729,7 +14804,7 @@
       <c r="X148" s="48"/>
       <c r="Y148" s="67"/>
     </row>
-    <row r="149" ht="16.5" spans="1:25">
+    <row r="149" ht="16.5" hidden="1" spans="1:25">
       <c r="A149" s="46">
         <v>147</v>
       </c>
@@ -14758,7 +14833,7 @@
       <c r="X149" s="48"/>
       <c r="Y149" s="67"/>
     </row>
-    <row r="150" ht="16.5" spans="1:25">
+    <row r="150" ht="16.5" hidden="1" spans="1:25">
       <c r="A150" s="46">
         <v>148</v>
       </c>
@@ -14768,7 +14843,7 @@
       <c r="E150" s="64"/>
       <c r="F150" s="64"/>
       <c r="G150" s="64"/>
-      <c r="H150" s="127"/>
+      <c r="H150" s="120"/>
       <c r="I150" s="63"/>
       <c r="J150" s="48"/>
       <c r="K150" s="65"/>
@@ -14787,7 +14862,7 @@
       <c r="X150" s="48"/>
       <c r="Y150" s="67"/>
     </row>
-    <row r="151" ht="16.5" spans="1:25">
+    <row r="151" ht="16.5" hidden="1" spans="1:25">
       <c r="A151" s="46">
         <v>149</v>
       </c>
@@ -14816,7 +14891,7 @@
       <c r="X151" s="48"/>
       <c r="Y151" s="67"/>
     </row>
-    <row r="152" ht="16.5" spans="1:25">
+    <row r="152" ht="16.5" hidden="1" spans="1:25">
       <c r="A152" s="46">
         <v>150</v>
       </c>
@@ -14845,17 +14920,17 @@
       <c r="X152" s="48"/>
       <c r="Y152" s="67"/>
     </row>
-    <row r="153" customHeight="1" spans="1:25">
+    <row r="153" hidden="1" customHeight="1" spans="1:25">
       <c r="A153" s="46">
         <v>151</v>
       </c>
       <c r="B153" s="48"/>
       <c r="C153" s="48"/>
       <c r="D153" s="63"/>
-      <c r="E153" s="127"/>
-      <c r="F153" s="127"/>
-      <c r="G153" s="127"/>
-      <c r="H153" s="127"/>
+      <c r="E153" s="120"/>
+      <c r="F153" s="120"/>
+      <c r="G153" s="120"/>
+      <c r="H153" s="120"/>
       <c r="I153" s="63"/>
       <c r="J153" s="48"/>
       <c r="K153" s="65"/>
@@ -14874,17 +14949,17 @@
       <c r="X153" s="48"/>
       <c r="Y153" s="67"/>
     </row>
-    <row r="154" customHeight="1" spans="1:25">
+    <row r="154" hidden="1" customHeight="1" spans="1:25">
       <c r="A154" s="46">
         <v>152</v>
       </c>
       <c r="B154" s="48"/>
       <c r="C154" s="48"/>
       <c r="D154" s="63"/>
-      <c r="E154" s="127"/>
-      <c r="F154" s="127"/>
-      <c r="G154" s="127"/>
-      <c r="H154" s="127"/>
+      <c r="E154" s="120"/>
+      <c r="F154" s="120"/>
+      <c r="G154" s="120"/>
+      <c r="H154" s="120"/>
       <c r="I154" s="63"/>
       <c r="J154" s="48"/>
       <c r="K154" s="65"/>
@@ -14903,17 +14978,17 @@
       <c r="X154" s="48"/>
       <c r="Y154" s="67"/>
     </row>
-    <row r="155" customHeight="1" spans="1:25">
+    <row r="155" hidden="1" customHeight="1" spans="1:25">
       <c r="A155" s="46">
         <v>153</v>
       </c>
       <c r="B155" s="48"/>
       <c r="C155" s="48"/>
       <c r="D155" s="63"/>
-      <c r="E155" s="127"/>
-      <c r="F155" s="127"/>
-      <c r="G155" s="127"/>
-      <c r="H155" s="127"/>
+      <c r="E155" s="120"/>
+      <c r="F155" s="120"/>
+      <c r="G155" s="120"/>
+      <c r="H155" s="120"/>
       <c r="I155" s="63"/>
       <c r="J155" s="48"/>
       <c r="K155" s="65"/>
@@ -14932,17 +15007,17 @@
       <c r="X155" s="48"/>
       <c r="Y155" s="67"/>
     </row>
-    <row r="156" customHeight="1" spans="1:25">
+    <row r="156" hidden="1" customHeight="1" spans="1:25">
       <c r="A156" s="46">
         <v>154</v>
       </c>
       <c r="B156" s="48"/>
       <c r="C156" s="48"/>
       <c r="D156" s="63"/>
-      <c r="E156" s="127"/>
-      <c r="F156" s="127"/>
-      <c r="G156" s="127"/>
-      <c r="H156" s="127"/>
+      <c r="E156" s="120"/>
+      <c r="F156" s="120"/>
+      <c r="G156" s="120"/>
+      <c r="H156" s="120"/>
       <c r="I156" s="63"/>
       <c r="J156" s="48"/>
       <c r="K156" s="65"/>
@@ -14961,17 +15036,17 @@
       <c r="X156" s="48"/>
       <c r="Y156" s="67"/>
     </row>
-    <row r="157" customHeight="1" spans="1:25">
+    <row r="157" hidden="1" customHeight="1" spans="1:25">
       <c r="A157" s="46">
         <v>155</v>
       </c>
       <c r="B157" s="48"/>
       <c r="C157" s="48"/>
       <c r="D157" s="63"/>
-      <c r="E157" s="127"/>
-      <c r="F157" s="127"/>
-      <c r="G157" s="127"/>
-      <c r="H157" s="127"/>
+      <c r="E157" s="120"/>
+      <c r="F157" s="120"/>
+      <c r="G157" s="120"/>
+      <c r="H157" s="120"/>
       <c r="I157" s="63"/>
       <c r="J157" s="48"/>
       <c r="K157" s="65"/>
@@ -14990,17 +15065,17 @@
       <c r="X157" s="48"/>
       <c r="Y157" s="67"/>
     </row>
-    <row r="158" customHeight="1" spans="1:25">
+    <row r="158" hidden="1" customHeight="1" spans="1:25">
       <c r="A158" s="46">
         <v>156</v>
       </c>
       <c r="B158" s="48"/>
       <c r="C158" s="48"/>
       <c r="D158" s="63"/>
-      <c r="E158" s="127"/>
-      <c r="F158" s="127"/>
-      <c r="G158" s="127"/>
-      <c r="H158" s="127"/>
+      <c r="E158" s="120"/>
+      <c r="F158" s="120"/>
+      <c r="G158" s="120"/>
+      <c r="H158" s="120"/>
       <c r="I158" s="63"/>
       <c r="J158" s="48"/>
       <c r="K158" s="65"/>
@@ -15019,17 +15094,17 @@
       <c r="X158" s="48"/>
       <c r="Y158" s="67"/>
     </row>
-    <row r="159" customHeight="1" spans="1:25">
+    <row r="159" hidden="1" customHeight="1" spans="1:25">
       <c r="A159" s="46">
         <v>157</v>
       </c>
       <c r="B159" s="48"/>
       <c r="C159" s="48"/>
       <c r="D159" s="63"/>
-      <c r="E159" s="127"/>
-      <c r="F159" s="127"/>
-      <c r="G159" s="127"/>
-      <c r="H159" s="127"/>
+      <c r="E159" s="120"/>
+      <c r="F159" s="120"/>
+      <c r="G159" s="120"/>
+      <c r="H159" s="120"/>
       <c r="I159" s="63"/>
       <c r="J159" s="48"/>
       <c r="K159" s="65"/>
@@ -15048,17 +15123,17 @@
       <c r="X159" s="48"/>
       <c r="Y159" s="67"/>
     </row>
-    <row r="160" customHeight="1" spans="1:25">
+    <row r="160" hidden="1" customHeight="1" spans="1:25">
       <c r="A160" s="46">
         <v>158</v>
       </c>
       <c r="B160" s="48"/>
       <c r="C160" s="48"/>
       <c r="D160" s="63"/>
-      <c r="E160" s="127"/>
-      <c r="F160" s="127"/>
-      <c r="G160" s="127"/>
-      <c r="H160" s="127"/>
+      <c r="E160" s="120"/>
+      <c r="F160" s="120"/>
+      <c r="G160" s="120"/>
+      <c r="H160" s="120"/>
       <c r="I160" s="63"/>
       <c r="J160" s="48"/>
       <c r="K160" s="65"/>
@@ -15077,10 +15152,16 @@
       <c r="X160" s="48"/>
       <c r="Y160" s="67"/>
     </row>
-    <row r="161" ht="13.5"/>
+    <row r="161" ht="13.5" hidden="1"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" insertColumns="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A2:Y161" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="15">
+      <customFilters>
+        <customFilter operator="equal" val="未结案"/>
+        <customFilter operator="equal" val="暂停"/>
+      </customFilters>
+    </filterColumn>
     <extLst/>
   </autoFilter>
   <mergeCells count="1">
@@ -15261,14 +15342,11 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B18">
       <formula1>"中东,北美,南美,拉美,南亚,东南亚,非洲,东欧,西欧,战略OEM,OBG"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X61 W62:X64 W1:X26 W28:X60 W75:X1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X61 W1:X26 W28:X60 W62:X64 W75:X1048576">
       <formula1>"有,无"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B64 B1:B17 B19:B49 B52:B61 B76:B1048576">
       <formula1>"中东,北美,南美,拉美,东欧,西欧,东南亚,南亚,战略OEM,非洲"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P71 P72 P73 P74 P1:P64 P65:P70 P75:P1048576">
-      <formula1>"结案,未结案,关闭,暂停"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B75">
       <formula1>"中东,北美,东南亚,南亚,东欧,西欧,拉美,南美,战略OEM,北非,中南非,OBG"</formula1>
@@ -15278,6 +15356,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O1:O64 O75:O1048576">
       <formula1>"客服,品质"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P$1:P$1048576">
+      <formula1>"结案,未结案,关闭,暂停"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U1:U60 U62:U64 U75:U77 U79:U1048576">
       <formula1>"电控,装配问题,裂管/漏氟,部品不良,包装破损,错漏发,噪音,结构不良,遥控器不良,外观不良,能力不足,漏水,压缩机,货柜漏水,散件订单设计,认证不符,其它,工艺设计,账物不符,标准差异,装柜问题,漏印商标,设计问题,设计优化"</formula1>

</xml_diff>

<commit_message>
data: 自动同步金山文档 2026-07-16 19:48
</commit_message>
<xml_diff>
--- a/2026年海外客户投诉台账.xlsx
+++ b/2026年海外客户投诉台账.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1290" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="487">
   <si>
     <t>2026年海外客诉台账</t>
   </si>
@@ -4989,6 +4989,39 @@
       </rPr>
       <t>【客户需求】分析调查和改善，并提供解决方案。</t>
     </r>
+  </si>
+  <si>
+    <t>洪都拉斯</t>
+  </si>
+  <si>
+    <t>【问题描述】洪都拉斯市场反馈24K外机售后问题，外机PCB没固定住，导致短路和其它不部件损坏，订单3000套，刚出售了21套就有4套机器出现这个问题，需要我们内部紧急核查是否是批量性的问题，给出不良原因分析和改善措施的答复报告
+【订单号】MO2509121190
+【订单机型】FTAC-24CSA-T13（室外机编码Z4U20103093158）
+【订单数量】3000
+【不良数量】4
+【不良率】19.04%
+【客户诉求】客户需要我们内部紧急核查是否是批量性的问题，给出不良原因分析和改善措施的答复报告</t>
+  </si>
+  <si>
+    <t>客户需要我们内部紧急核查是否是批量性的问题，给出不良原因分析和改善措施的答复报告</t>
+  </si>
+  <si>
+    <t>制造主因：飞机钉未卡到位，PCB松脱后在运输/运行振动下与周边金属件干涉短路。
+工艺次因：员工反馈难装配，工艺未评估异常影响，未启动PQE评估。
+质量次因：飞机钉未卡到位时PCB明显晃动，检验未识别，员工质量意识不足。</t>
+  </si>
+  <si>
+    <t>装配加严：飞机钉安装后执行回拔确认，插线岗位互检PCB固定状态。
+标准固化：编制飞机钉装配及来料检验作业指导书，明确"卡入到位、无松脱、无晃动"标准。
+培训强化：电控班开展飞机钉装配要点、回拔动作及互检要求专项培训。
+检验升级：PQC巡检频次由1小时/次缩短至30分钟/次；OQC增加PCB固定可靠性拍照检点。
+人员管控：排查电控班人员编制，落实定岗，提升待遇。</t>
+  </si>
+  <si>
+    <t>制造中心/制程品管部</t>
+  </si>
+  <si>
+    <t>待人员出差现场抽检机器确认是否存在批量问题</t>
   </si>
   <si>
     <t>2026海外市场退回件报表</t>
@@ -5205,13 +5238,13 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
@@ -6389,7 +6422,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="124">
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6706,9 +6739,6 @@
     <xf numFmtId="14" fontId="18" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="18" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="10" fontId="18" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6730,9 +6760,6 @@
     <xf numFmtId="14" fontId="18" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="18" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="10" fontId="18" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6746,6 +6773,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="22" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6758,7 +6788,7 @@
     <xf numFmtId="176" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6779,19 +6809,19 @@
     <xf numFmtId="176" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6947,7 +6977,7 @@
 <file path=xl/woinfos.xml><?xml version="1.0" encoding="utf-8"?>
 <woInfos xmlns="https://web.wps.cn/et/2018/main" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <bookInfo cellCmpFml="4" dbFileVersion="0" changeLogVersion="0">
-    <open main="58" threadCnt="1"/>
+    <open main="48" threadCnt="1"/>
     <sheetInfos>
       <sheetInfo cellCmpFml="4" sheetStid="3">
         <open main="5" threadCnt="1"/>
@@ -7246,7 +7276,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1" codeName="Sheet1">
+  <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Y161"/>
@@ -7441,7 +7471,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" s="24" customFormat="1" ht="128.25" hidden="1" spans="1:25">
+    <row r="4" s="24" customFormat="1" ht="128.25" spans="1:25">
       <c r="A4" s="46">
         <v>2</v>
       </c>
@@ -7513,7 +7543,7 @@
       <c r="X4" s="47"/>
       <c r="Y4" s="56"/>
     </row>
-    <row r="5" s="25" customFormat="1" ht="99.75" hidden="1" spans="1:25">
+    <row r="5" s="25" customFormat="1" ht="99.75" spans="1:25">
       <c r="A5" s="46">
         <v>3</v>
       </c>
@@ -7589,7 +7619,7 @@
       </c>
       <c r="Y5" s="61"/>
     </row>
-    <row r="6" s="25" customFormat="1" ht="128.25" hidden="1" spans="1:25">
+    <row r="6" s="25" customFormat="1" ht="128.25" spans="1:25">
       <c r="A6" s="46">
         <v>4</v>
       </c>
@@ -7665,7 +7695,7 @@
       </c>
       <c r="Y6" s="61"/>
     </row>
-    <row r="7" s="25" customFormat="1" ht="285" hidden="1" spans="1:25">
+    <row r="7" s="25" customFormat="1" ht="285" spans="1:25">
       <c r="A7" s="46">
         <v>5</v>
       </c>
@@ -7739,7 +7769,7 @@
       <c r="X7" s="60"/>
       <c r="Y7" s="61"/>
     </row>
-    <row r="8" s="25" customFormat="1" ht="117.95" hidden="1" customHeight="1" spans="1:25">
+    <row r="8" s="25" customFormat="1" ht="117.95" customHeight="1" spans="1:25">
       <c r="A8" s="46">
         <v>6</v>
       </c>
@@ -7813,7 +7843,7 @@
       <c r="X8" s="60"/>
       <c r="Y8" s="61"/>
     </row>
-    <row r="9" s="25" customFormat="1" ht="128.25" hidden="1" spans="1:25">
+    <row r="9" s="25" customFormat="1" ht="128.25" spans="1:25">
       <c r="A9" s="46">
         <v>7</v>
       </c>
@@ -7889,7 +7919,7 @@
       </c>
       <c r="Y9" s="61"/>
     </row>
-    <row r="10" ht="156.75" hidden="1" spans="1:25">
+    <row r="10" ht="156.75" spans="1:25">
       <c r="A10" s="46">
         <v>8</v>
       </c>
@@ -7967,7 +7997,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="11" ht="99.75" hidden="1" spans="1:25">
+    <row r="11" ht="99.75" spans="1:25">
       <c r="A11" s="46">
         <v>9</v>
       </c>
@@ -8041,7 +8071,7 @@
       </c>
       <c r="Y11" s="67"/>
     </row>
-    <row r="12" ht="99.75" hidden="1" spans="1:25">
+    <row r="12" ht="99.75" spans="1:25">
       <c r="A12" s="46">
         <v>10</v>
       </c>
@@ -8117,7 +8147,7 @@
       </c>
       <c r="Y12" s="67"/>
     </row>
-    <row r="13" ht="142.5" hidden="1" spans="1:25">
+    <row r="13" ht="142.5" spans="1:25">
       <c r="A13" s="46">
         <v>11</v>
       </c>
@@ -8195,7 +8225,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="14" ht="114" hidden="1" spans="1:25">
+    <row r="14" ht="114" spans="1:25">
       <c r="A14" s="46">
         <v>12</v>
       </c>
@@ -8273,7 +8303,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="15" ht="128.25" hidden="1" spans="1:25">
+    <row r="15" ht="128.25" spans="1:25">
       <c r="A15" s="46">
         <v>13</v>
       </c>
@@ -8343,7 +8373,7 @@
       </c>
       <c r="Y15" s="67"/>
     </row>
-    <row r="16" ht="114" hidden="1" spans="1:25">
+    <row r="16" ht="114" spans="1:25">
       <c r="A16" s="46">
         <v>14</v>
       </c>
@@ -8421,7 +8451,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="17" ht="114" hidden="1" spans="1:25">
+    <row r="17" ht="114" spans="1:25">
       <c r="A17" s="46">
         <v>15</v>
       </c>
@@ -8495,7 +8525,7 @@
       <c r="X17" s="48"/>
       <c r="Y17" s="67"/>
     </row>
-    <row r="18" ht="150" hidden="1" customHeight="1" spans="1:25">
+    <row r="18" ht="150" customHeight="1" spans="1:25">
       <c r="A18" s="46">
         <v>16</v>
       </c>
@@ -8569,7 +8599,7 @@
       </c>
       <c r="Y18" s="67"/>
     </row>
-    <row r="19" ht="99.75" hidden="1" spans="1:25">
+    <row r="19" ht="99.75" spans="1:25">
       <c r="A19" s="46">
         <v>17</v>
       </c>
@@ -8643,7 +8673,7 @@
       </c>
       <c r="Y19" s="67"/>
     </row>
-    <row r="20" ht="199.5" hidden="1" spans="1:25">
+    <row r="20" ht="199.5" spans="1:25">
       <c r="A20" s="46">
         <v>18</v>
       </c>
@@ -8717,7 +8747,7 @@
       <c r="X20" s="48"/>
       <c r="Y20" s="67"/>
     </row>
-    <row r="21" ht="99.75" hidden="1" spans="1:25">
+    <row r="21" ht="99.75" spans="1:25">
       <c r="A21" s="46">
         <v>19</v>
       </c>
@@ -8791,7 +8821,7 @@
       <c r="X21" s="48"/>
       <c r="Y21" s="67"/>
     </row>
-    <row r="22" ht="185.25" hidden="1" spans="1:25">
+    <row r="22" ht="185.25" spans="1:25">
       <c r="A22" s="46">
         <v>20</v>
       </c>
@@ -8865,7 +8895,7 @@
       <c r="X22" s="48"/>
       <c r="Y22" s="67"/>
     </row>
-    <row r="23" ht="85.5" hidden="1" customHeight="1" spans="1:25">
+    <row r="23" ht="85.5" customHeight="1" spans="1:25">
       <c r="A23" s="46">
         <v>21</v>
       </c>
@@ -8941,7 +8971,7 @@
       </c>
       <c r="Y23" s="67"/>
     </row>
-    <row r="24" ht="156.75" hidden="1" spans="1:25">
+    <row r="24" ht="156.75" spans="1:25">
       <c r="A24" s="46">
         <v>22</v>
       </c>
@@ -9019,7 +9049,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="25" ht="99.75" hidden="1" spans="1:25">
+    <row r="25" ht="99.75" spans="1:25">
       <c r="A25" s="46">
         <v>23</v>
       </c>
@@ -9087,7 +9117,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="26" ht="297" hidden="1" spans="1:25">
+    <row r="26" ht="297" spans="1:25">
       <c r="A26" s="46">
         <v>24</v>
       </c>
@@ -9160,7 +9190,7 @@
       </c>
       <c r="X26" s="48"/>
     </row>
-    <row r="27" ht="132" hidden="1" spans="1:25">
+    <row r="27" ht="132" spans="1:25">
       <c r="A27" s="46">
         <v>25</v>
       </c>
@@ -9235,7 +9265,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" ht="148.5" hidden="1" spans="1:25">
+    <row r="28" ht="148.5" spans="1:25">
       <c r="A28" s="46">
         <v>26</v>
       </c>
@@ -9308,7 +9338,7 @@
       </c>
       <c r="X28" s="48"/>
     </row>
-    <row r="29" ht="247.5" hidden="1" spans="1:25">
+    <row r="29" ht="247.5" spans="1:25">
       <c r="A29" s="46">
         <v>27</v>
       </c>
@@ -9381,7 +9411,7 @@
       </c>
       <c r="X29" s="48"/>
     </row>
-    <row r="30" customFormat="1" ht="128.25" hidden="1" spans="1:25">
+    <row r="30" customFormat="1" ht="128.25" spans="1:25">
       <c r="A30" s="46">
         <v>28</v>
       </c>
@@ -9455,7 +9485,7 @@
       </c>
       <c r="Y30" s="67"/>
     </row>
-    <row r="31" customFormat="1" ht="128.25" hidden="1" spans="1:25">
+    <row r="31" customFormat="1" ht="128.25" spans="1:25">
       <c r="A31" s="46">
         <v>29</v>
       </c>
@@ -9525,7 +9555,7 @@
       <c r="X31" s="48"/>
       <c r="Y31" s="67"/>
     </row>
-    <row r="32" customFormat="1" ht="142.5" hidden="1" spans="1:25">
+    <row r="32" customFormat="1" ht="142.5" spans="1:25">
       <c r="A32" s="46">
         <v>30</v>
       </c>
@@ -9601,7 +9631,7 @@
       </c>
       <c r="Y32" s="67"/>
     </row>
-    <row r="33" customFormat="1" ht="114" hidden="1" spans="1:25">
+    <row r="33" customFormat="1" ht="114" spans="1:25">
       <c r="A33" s="46">
         <v>31</v>
       </c>
@@ -9665,7 +9695,7 @@
       <c r="X33" s="48"/>
       <c r="Y33" s="67"/>
     </row>
-    <row r="34" ht="114" hidden="1" spans="1:25">
+    <row r="34" ht="114" spans="1:25">
       <c r="A34" s="46">
         <v>32</v>
       </c>
@@ -9741,7 +9771,7 @@
       </c>
       <c r="Y34" s="67"/>
     </row>
-    <row r="35" ht="142.5" hidden="1" spans="1:25">
+    <row r="35" ht="142.5" spans="1:25">
       <c r="A35" s="46">
         <v>33</v>
       </c>
@@ -9817,7 +9847,7 @@
       </c>
       <c r="Y35" s="67"/>
     </row>
-    <row r="36" ht="99.75" hidden="1" spans="1:25">
+    <row r="36" ht="99.75" spans="1:25">
       <c r="A36" s="46">
         <v>34</v>
       </c>
@@ -9893,7 +9923,7 @@
       </c>
       <c r="Y36" s="67"/>
     </row>
-    <row r="37" customFormat="1" ht="142.5" hidden="1" spans="1:25">
+    <row r="37" customFormat="1" ht="142.5" spans="1:25">
       <c r="A37" s="46">
         <v>35</v>
       </c>
@@ -9971,7 +10001,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="38" ht="148.5" hidden="1" spans="1:25">
+    <row r="38" ht="148.5" spans="1:25">
       <c r="A38" s="46">
         <v>36</v>
       </c>
@@ -10047,7 +10077,7 @@
       </c>
       <c r="Y38" s="67"/>
     </row>
-    <row r="39" ht="142.5" hidden="1" spans="1:25">
+    <row r="39" ht="142.5" spans="1:25">
       <c r="A39" s="46">
         <v>37</v>
       </c>
@@ -10123,7 +10153,7 @@
       </c>
       <c r="Y39" s="67"/>
     </row>
-    <row r="40" ht="342" hidden="1" spans="1:25">
+    <row r="40" ht="342" spans="1:25">
       <c r="A40" s="46">
         <v>38</v>
       </c>
@@ -10251,7 +10281,7 @@
       <c r="X41" s="48"/>
       <c r="Y41" s="67"/>
     </row>
-    <row r="42" ht="171" hidden="1" spans="1:25">
+    <row r="42" ht="171" spans="1:25">
       <c r="A42" s="46">
         <v>40</v>
       </c>
@@ -10325,7 +10355,7 @@
       <c r="X42" s="48"/>
       <c r="Y42" s="67"/>
     </row>
-    <row r="43" ht="342" hidden="1" spans="1:25">
+    <row r="43" ht="342" spans="1:25">
       <c r="A43" s="46">
         <v>41</v>
       </c>
@@ -10399,7 +10429,7 @@
       <c r="X43" s="48"/>
       <c r="Y43" s="67"/>
     </row>
-    <row r="44" ht="153" hidden="1" customHeight="1" spans="1:25">
+    <row r="44" ht="153" customHeight="1" spans="1:25">
       <c r="A44" s="46">
         <v>42</v>
       </c>
@@ -10471,7 +10501,7 @@
       <c r="X44" s="48"/>
       <c r="Y44" s="67"/>
     </row>
-    <row r="45" ht="163.5" hidden="1" customHeight="1" spans="1:25">
+    <row r="45" ht="163.5" customHeight="1" spans="1:25">
       <c r="A45" s="46">
         <v>43</v>
       </c>
@@ -10545,7 +10575,7 @@
       <c r="X45" s="48"/>
       <c r="Y45" s="67"/>
     </row>
-    <row r="46" ht="299.25" hidden="1" spans="1:25">
+    <row r="46" ht="299.25" spans="1:25">
       <c r="A46" s="46">
         <v>44</v>
       </c>
@@ -10619,7 +10649,7 @@
       <c r="X46" s="48"/>
       <c r="Y46" s="67"/>
     </row>
-    <row r="47" ht="149.25" hidden="1" customHeight="1" spans="1:25">
+    <row r="47" ht="149.25" customHeight="1" spans="1:25">
       <c r="A47" s="46">
         <v>45</v>
       </c>
@@ -10695,7 +10725,7 @@
       </c>
       <c r="Y47" s="67"/>
     </row>
-    <row r="48" ht="149.25" hidden="1" customHeight="1" spans="1:25">
+    <row r="48" ht="149.25" customHeight="1" spans="1:25">
       <c r="A48" s="46">
         <v>46</v>
       </c>
@@ -10773,7 +10803,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="49" ht="149.25" hidden="1" customHeight="1" spans="1:25">
+    <row r="49" ht="149.25" customHeight="1" spans="1:25">
       <c r="A49" s="46">
         <v>47</v>
       </c>
@@ -10849,7 +10879,7 @@
       </c>
       <c r="Y49" s="67"/>
     </row>
-    <row r="50" ht="114" hidden="1" spans="1:25">
+    <row r="50" ht="114" spans="1:25">
       <c r="A50" s="46">
         <v>48</v>
       </c>
@@ -10925,7 +10955,7 @@
       </c>
       <c r="Y50" s="67"/>
     </row>
-    <row r="51" ht="114" hidden="1" spans="1:25">
+    <row r="51" ht="114" spans="1:25">
       <c r="A51" s="46">
         <v>49</v>
       </c>
@@ -10999,7 +11029,7 @@
       <c r="X51" s="48"/>
       <c r="Y51" s="67"/>
     </row>
-    <row r="52" ht="128.25" hidden="1" spans="1:25">
+    <row r="52" ht="128.25" spans="1:25">
       <c r="A52" s="46">
         <v>50</v>
       </c>
@@ -11073,7 +11103,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="53" ht="384.75" hidden="1" spans="1:25">
+    <row r="53" ht="384.75" spans="1:25">
       <c r="A53" s="46">
         <v>51</v>
       </c>
@@ -11147,7 +11177,7 @@
       <c r="X53" s="48"/>
       <c r="Y53" s="67"/>
     </row>
-    <row r="54" ht="136.5" hidden="1" customHeight="1" spans="1:25">
+    <row r="54" ht="136.5" customHeight="1" spans="1:25">
       <c r="A54" s="46">
         <v>52</v>
       </c>
@@ -11219,7 +11249,7 @@
       </c>
       <c r="Y54" s="67"/>
     </row>
-    <row r="55" ht="136.5" hidden="1" customHeight="1" spans="1:25">
+    <row r="55" ht="136.5" customHeight="1" spans="1:25">
       <c r="A55" s="46">
         <v>53</v>
       </c>
@@ -11293,7 +11323,7 @@
       <c r="X55" s="48"/>
       <c r="Y55" s="67"/>
     </row>
-    <row r="56" ht="85.5" hidden="1" spans="1:25">
+    <row r="56" ht="85.5" spans="1:25">
       <c r="A56" s="46">
         <v>54</v>
       </c>
@@ -11369,7 +11399,7 @@
       </c>
       <c r="Y56" s="67"/>
     </row>
-    <row r="57" ht="99.75" hidden="1" spans="1:25">
+    <row r="57" ht="99.75" spans="1:25">
       <c r="A57" s="46">
         <v>55</v>
       </c>
@@ -11445,7 +11475,7 @@
       </c>
       <c r="Y57" s="67"/>
     </row>
-    <row r="58" ht="99.75" hidden="1" spans="1:25">
+    <row r="58" ht="99.75" spans="1:25">
       <c r="A58" s="46">
         <v>56</v>
       </c>
@@ -11523,7 +11553,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="59" ht="159" hidden="1" customHeight="1" spans="1:25">
+    <row r="59" ht="159" customHeight="1" spans="1:25">
       <c r="A59" s="46">
         <v>57</v>
       </c>
@@ -11653,7 +11683,7 @@
       <c r="X60" s="48"/>
       <c r="Y60" s="67"/>
     </row>
-    <row r="61" ht="132" hidden="1" customHeight="1" spans="1:25">
+    <row r="61" ht="132" customHeight="1" spans="1:25">
       <c r="A61" s="46">
         <v>59</v>
       </c>
@@ -11721,7 +11751,7 @@
       <c r="X61" s="48"/>
       <c r="Y61" s="67"/>
     </row>
-    <row r="62" ht="132" hidden="1" spans="1:25">
+    <row r="62" ht="132" spans="1:25">
       <c r="A62" s="46">
         <v>60</v>
       </c>
@@ -11797,7 +11827,7 @@
       </c>
       <c r="Y62" s="67"/>
     </row>
-    <row r="63" ht="132" hidden="1" spans="1:25">
+    <row r="63" ht="132" spans="1:25">
       <c r="A63" s="46">
         <v>61</v>
       </c>
@@ -11873,7 +11903,7 @@
       </c>
       <c r="Y63" s="67"/>
     </row>
-    <row r="64" ht="199.15" hidden="1" customHeight="1" spans="1:25">
+    <row r="64" ht="199.15" customHeight="1" spans="1:25">
       <c r="A64" s="46">
         <v>62</v>
       </c>
@@ -11951,7 +11981,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="65" ht="99.75" hidden="1" spans="1:25">
+    <row r="65" ht="99.75" spans="1:25">
       <c r="A65" s="46">
         <v>63</v>
       </c>
@@ -12027,7 +12057,7 @@
       </c>
       <c r="Y65" s="89"/>
     </row>
-    <row r="66" ht="142.5" hidden="1" spans="1:25">
+    <row r="66" ht="142.5" spans="1:25">
       <c r="A66" s="46">
         <v>64</v>
       </c>
@@ -12103,7 +12133,7 @@
       </c>
       <c r="Y66" s="89"/>
     </row>
-    <row r="67" ht="128.25" hidden="1" spans="1:25">
+    <row r="67" ht="128.25" spans="1:25">
       <c r="A67" s="46">
         <v>65</v>
       </c>
@@ -12173,7 +12203,7 @@
       <c r="X67" s="86"/>
       <c r="Y67" s="89"/>
     </row>
-    <row r="68" ht="156.75" hidden="1" spans="1:25">
+    <row r="68" ht="156.75" spans="1:25">
       <c r="A68" s="46">
         <v>66</v>
       </c>
@@ -12251,7 +12281,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="69" ht="96" hidden="1" customHeight="1" spans="1:25">
+    <row r="69" ht="96" customHeight="1" spans="1:25">
       <c r="A69" s="46">
         <v>67</v>
       </c>
@@ -12329,7 +12359,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="70" ht="84.75" hidden="1" customHeight="1" spans="1:25">
+    <row r="70" ht="84.75" customHeight="1" spans="1:25">
       <c r="A70" s="46">
         <v>68</v>
       </c>
@@ -12465,7 +12495,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="72" ht="108" hidden="1" customHeight="1" spans="1:25">
+    <row r="72" ht="108" customHeight="1" spans="1:25">
       <c r="A72" s="46">
         <v>70</v>
       </c>
@@ -12537,7 +12567,7 @@
       <c r="X72" s="86"/>
       <c r="Y72" s="89"/>
     </row>
-    <row r="73" ht="145.5" hidden="1" customHeight="1" spans="1:25">
+    <row r="73" ht="145.5" customHeight="1" spans="1:25">
       <c r="A73" s="46">
         <v>71</v>
       </c>
@@ -12556,7 +12586,8 @@
       <c r="F73" s="95">
         <v>46227</v>
       </c>
-      <c r="G73" s="96">
+      <c r="G73" s="50">
+        <f>WORKDAY(F73,-3)</f>
         <v>46224</v>
       </c>
       <c r="H73" s="95">
@@ -12568,13 +12599,13 @@
       <c r="J73" s="81" t="s">
         <v>284</v>
       </c>
-      <c r="K73" s="97" t="s">
+      <c r="K73" s="96" t="s">
         <v>44</v>
       </c>
-      <c r="L73" s="98" t="s">
+      <c r="L73" s="97" t="s">
         <v>459</v>
       </c>
-      <c r="M73" s="98" t="s">
+      <c r="M73" s="97" t="s">
         <v>460</v>
       </c>
       <c r="N73" s="81" t="s">
@@ -12586,8 +12617,8 @@
       <c r="P73" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="Q73" s="98"/>
-      <c r="R73" s="98" t="s">
+      <c r="Q73" s="97"/>
+      <c r="R73" s="97" t="s">
         <v>461</v>
       </c>
       <c r="S73" s="80" t="s">
@@ -12606,103 +12637,153 @@
         <v>50</v>
       </c>
       <c r="X73" s="81"/>
-      <c r="Y73" s="99"/>
+      <c r="Y73" s="98"/>
     </row>
     <row r="74" ht="142.5" customHeight="1" spans="1:25">
       <c r="A74" s="46">
         <v>72</v>
       </c>
-      <c r="B74" s="100" t="s">
+      <c r="B74" s="99" t="s">
         <v>72</v>
       </c>
-      <c r="C74" s="101" t="s">
+      <c r="C74" s="100" t="s">
         <v>283</v>
       </c>
-      <c r="D74" s="102" t="s">
+      <c r="D74" s="101" t="s">
         <v>28</v>
       </c>
-      <c r="E74" s="103">
+      <c r="E74" s="102">
         <v>46216</v>
       </c>
-      <c r="F74" s="103">
+      <c r="F74" s="102">
         <v>46227</v>
       </c>
-      <c r="G74" s="104">
+      <c r="G74" s="50">
+        <f>WORKDAY(F74,-3)</f>
         <v>46224</v>
       </c>
-      <c r="H74" s="103"/>
-      <c r="I74" s="102"/>
-      <c r="J74" s="101" t="s">
+      <c r="H74" s="102"/>
+      <c r="I74" s="101"/>
+      <c r="J74" s="100" t="s">
         <v>284</v>
       </c>
-      <c r="K74" s="105" t="s">
+      <c r="K74" s="103" t="s">
         <v>44</v>
       </c>
-      <c r="L74" s="106" t="s">
+      <c r="L74" s="104" t="s">
         <v>463</v>
       </c>
-      <c r="M74" s="106" t="s">
+      <c r="M74" s="104" t="s">
         <v>460</v>
       </c>
-      <c r="N74" s="101" t="s">
+      <c r="N74" s="100" t="s">
         <v>42</v>
       </c>
-      <c r="O74" s="101" t="s">
+      <c r="O74" s="100" t="s">
         <v>33</v>
       </c>
       <c r="P74" s="48" t="s">
         <v>291</v>
       </c>
-      <c r="Q74" s="106"/>
-      <c r="R74" s="106"/>
-      <c r="S74" s="107"/>
-      <c r="T74" s="101"/>
-      <c r="U74" s="101"/>
-      <c r="V74" s="101"/>
-      <c r="W74" s="101"/>
-      <c r="X74" s="101"/>
-      <c r="Y74" s="108"/>
-    </row>
-    <row r="75" ht="142.5" hidden="1" customHeight="1" spans="1:25">
+      <c r="Q74" s="104"/>
+      <c r="R74" s="104"/>
+      <c r="S74" s="105"/>
+      <c r="T74" s="100"/>
+      <c r="U74" s="100"/>
+      <c r="V74" s="100"/>
+      <c r="W74" s="100"/>
+      <c r="X74" s="100"/>
+      <c r="Y74" s="106"/>
+    </row>
+    <row r="75" ht="142.5" customHeight="1" spans="1:25">
       <c r="A75" s="46">
         <v>73</v>
       </c>
-      <c r="B75" s="109"/>
-      <c r="C75" s="109"/>
-      <c r="D75" s="63"/>
-      <c r="E75" s="110"/>
-      <c r="F75" s="110"/>
-      <c r="G75" s="110"/>
-      <c r="H75" s="110"/>
-      <c r="I75" s="63"/>
-      <c r="J75" s="48"/>
-      <c r="K75" s="65"/>
-      <c r="L75" s="53"/>
-      <c r="M75" s="53"/>
-      <c r="N75" s="48"/>
-      <c r="O75" s="48"/>
-      <c r="P75" s="48"/>
-      <c r="Q75" s="53"/>
-      <c r="R75" s="53"/>
-      <c r="S75" s="66"/>
-      <c r="T75" s="48"/>
-      <c r="U75" s="48"/>
-      <c r="V75" s="48"/>
-      <c r="W75" s="48"/>
-      <c r="X75" s="48"/>
-      <c r="Y75" s="67"/>
-    </row>
-    <row r="76" ht="141.75" hidden="1" customHeight="1" spans="1:25">
+      <c r="B75" s="107" t="s">
+        <v>266</v>
+      </c>
+      <c r="C75" s="108" t="s">
+        <v>464</v>
+      </c>
+      <c r="D75" s="63" t="s">
+        <v>28</v>
+      </c>
+      <c r="E75" s="109">
+        <v>46209</v>
+      </c>
+      <c r="F75" s="109">
+        <v>46220</v>
+      </c>
+      <c r="G75" s="50">
+        <f>WORKDAY(F75,-3)</f>
+        <v>46217</v>
+      </c>
+      <c r="H75" s="109">
+        <v>46219</v>
+      </c>
+      <c r="I75" s="79" t="s">
+        <v>369</v>
+      </c>
+      <c r="J75" s="48" t="s">
+        <v>284</v>
+      </c>
+      <c r="K75" s="65">
+        <v>0.1904</v>
+      </c>
+      <c r="L75" s="68" t="s">
+        <v>465</v>
+      </c>
+      <c r="M75" s="68" t="s">
+        <v>466</v>
+      </c>
+      <c r="N75" s="85" t="s">
+        <v>102</v>
+      </c>
+      <c r="O75" s="48" t="s">
+        <v>59</v>
+      </c>
+      <c r="P75" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q75" s="68" t="s">
+        <v>35</v>
+      </c>
+      <c r="R75" s="68" t="s">
+        <v>467</v>
+      </c>
+      <c r="S75" s="84" t="s">
+        <v>468</v>
+      </c>
+      <c r="T75" s="85" t="s">
+        <v>469</v>
+      </c>
+      <c r="U75" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="V75" s="85" t="s">
+        <v>64</v>
+      </c>
+      <c r="W75" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="X75" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y75" s="68" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="76" ht="141.75" customHeight="1" spans="1:25">
       <c r="A76" s="46">
         <v>74</v>
       </c>
       <c r="B76" s="48"/>
       <c r="C76" s="48"/>
       <c r="D76" s="63"/>
-      <c r="E76" s="110"/>
-      <c r="F76" s="110"/>
-      <c r="G76" s="110"/>
-      <c r="H76" s="110"/>
+      <c r="E76" s="109"/>
+      <c r="F76" s="109"/>
+      <c r="G76" s="109"/>
+      <c r="H76" s="109"/>
       <c r="I76" s="63"/>
       <c r="J76" s="48"/>
       <c r="K76" s="65"/>
@@ -12721,7 +12802,7 @@
       <c r="X76" s="48"/>
       <c r="Y76" s="67"/>
     </row>
-    <row r="77" ht="141.75" hidden="1" customHeight="1" spans="1:25">
+    <row r="77" ht="141.75" customHeight="1" spans="1:25">
       <c r="A77" s="46">
         <v>75</v>
       </c>
@@ -12750,7 +12831,7 @@
       <c r="X77" s="48"/>
       <c r="Y77" s="67"/>
     </row>
-    <row r="78" ht="16.5" hidden="1" spans="1:25">
+    <row r="78" ht="16.5" spans="1:25">
       <c r="A78" s="46">
         <v>76</v>
       </c>
@@ -12774,12 +12855,12 @@
       <c r="S78" s="53"/>
       <c r="T78" s="66"/>
       <c r="U78" s="48"/>
-      <c r="V78" s="111"/>
+      <c r="V78" s="110"/>
       <c r="W78" s="48"/>
       <c r="X78" s="48"/>
       <c r="Y78" s="67"/>
     </row>
-    <row r="79" ht="16.5" hidden="1" spans="1:25">
+    <row r="79" ht="16.5" spans="1:25">
       <c r="A79" s="46">
         <v>77</v>
       </c>
@@ -12808,7 +12889,7 @@
       <c r="X79" s="48"/>
       <c r="Y79" s="67"/>
     </row>
-    <row r="80" ht="16.5" hidden="1" spans="1:25">
+    <row r="80" ht="16.5" spans="1:25">
       <c r="A80" s="46">
         <v>78</v>
       </c>
@@ -12837,7 +12918,7 @@
       <c r="X80" s="48"/>
       <c r="Y80" s="67"/>
     </row>
-    <row r="81" ht="16.5" hidden="1" spans="1:25">
+    <row r="81" ht="16.5" spans="1:25">
       <c r="A81" s="46">
         <v>79</v>
       </c>
@@ -12866,7 +12947,7 @@
       <c r="X81" s="48"/>
       <c r="Y81" s="67"/>
     </row>
-    <row r="82" ht="16.5" hidden="1" spans="1:25">
+    <row r="82" ht="16.5" spans="1:25">
       <c r="A82" s="46">
         <v>80</v>
       </c>
@@ -12895,7 +12976,7 @@
       <c r="X82" s="48"/>
       <c r="Y82" s="67"/>
     </row>
-    <row r="83" ht="16.5" hidden="1" spans="1:25">
+    <row r="83" ht="16.5" spans="1:25">
       <c r="A83" s="46">
         <v>81</v>
       </c>
@@ -12924,7 +13005,7 @@
       <c r="X83" s="48"/>
       <c r="Y83" s="67"/>
     </row>
-    <row r="84" ht="16.5" hidden="1" spans="1:25">
+    <row r="84" ht="16.5" spans="1:25">
       <c r="A84" s="46">
         <v>82</v>
       </c>
@@ -12953,7 +13034,7 @@
       <c r="X84" s="48"/>
       <c r="Y84" s="67"/>
     </row>
-    <row r="85" ht="16.5" hidden="1" spans="1:25">
+    <row r="85" ht="16.5" spans="1:25">
       <c r="A85" s="46">
         <v>83</v>
       </c>
@@ -12982,7 +13063,7 @@
       <c r="X85" s="48"/>
       <c r="Y85" s="67"/>
     </row>
-    <row r="86" ht="16.5" hidden="1" spans="1:25">
+    <row r="86" ht="16.5" spans="1:25">
       <c r="A86" s="46">
         <v>84</v>
       </c>
@@ -13011,7 +13092,7 @@
       <c r="X86" s="48"/>
       <c r="Y86" s="67"/>
     </row>
-    <row r="87" ht="16.5" hidden="1" spans="1:25">
+    <row r="87" ht="16.5" spans="1:25">
       <c r="A87" s="46">
         <v>85</v>
       </c>
@@ -13040,7 +13121,7 @@
       <c r="X87" s="48"/>
       <c r="Y87" s="67"/>
     </row>
-    <row r="88" ht="16.5" hidden="1" spans="1:25">
+    <row r="88" ht="16.5" spans="1:25">
       <c r="A88" s="46">
         <v>86</v>
       </c>
@@ -13069,7 +13150,7 @@
       <c r="X88" s="48"/>
       <c r="Y88" s="67"/>
     </row>
-    <row r="89" ht="16.5" hidden="1" spans="1:25">
+    <row r="89" ht="16.5" spans="1:25">
       <c r="A89" s="46">
         <v>87</v>
       </c>
@@ -13098,7 +13179,7 @@
       <c r="X89" s="48"/>
       <c r="Y89" s="67"/>
     </row>
-    <row r="90" ht="16.5" hidden="1" spans="1:25">
+    <row r="90" ht="16.5" spans="1:25">
       <c r="A90" s="46">
         <v>88</v>
       </c>
@@ -13127,7 +13208,7 @@
       <c r="X90" s="48"/>
       <c r="Y90" s="67"/>
     </row>
-    <row r="91" ht="16.5" hidden="1" spans="1:25">
+    <row r="91" ht="16.5" spans="1:25">
       <c r="A91" s="46">
         <v>89</v>
       </c>
@@ -13156,7 +13237,7 @@
       <c r="X91" s="48"/>
       <c r="Y91" s="67"/>
     </row>
-    <row r="92" ht="16.5" hidden="1" spans="1:25">
+    <row r="92" ht="16.5" spans="1:25">
       <c r="A92" s="46">
         <v>90</v>
       </c>
@@ -13185,7 +13266,7 @@
       <c r="X92" s="48"/>
       <c r="Y92" s="67"/>
     </row>
-    <row r="93" ht="16.5" hidden="1" spans="1:25">
+    <row r="93" ht="16.5" spans="1:25">
       <c r="A93" s="46">
         <v>91</v>
       </c>
@@ -13214,7 +13295,7 @@
       <c r="X93" s="48"/>
       <c r="Y93" s="67"/>
     </row>
-    <row r="94" ht="16.5" hidden="1" spans="1:25">
+    <row r="94" ht="16.5" spans="1:25">
       <c r="A94" s="46">
         <v>92</v>
       </c>
@@ -13243,7 +13324,7 @@
       <c r="X94" s="48"/>
       <c r="Y94" s="67"/>
     </row>
-    <row r="95" ht="99.75" hidden="1" customHeight="1" spans="1:25">
+    <row r="95" ht="99.75" customHeight="1" spans="1:25">
       <c r="A95" s="46">
         <v>93</v>
       </c>
@@ -13272,7 +13353,7 @@
       <c r="X95" s="48"/>
       <c r="Y95" s="67"/>
     </row>
-    <row r="96" ht="146.25" hidden="1" customHeight="1" spans="1:25">
+    <row r="96" ht="146.25" customHeight="1" spans="1:25">
       <c r="A96" s="46">
         <v>94</v>
       </c>
@@ -13301,7 +13382,7 @@
       <c r="X96" s="48"/>
       <c r="Y96" s="67"/>
     </row>
-    <row r="97" ht="16.5" hidden="1" spans="1:25">
+    <row r="97" ht="16.5" spans="1:25">
       <c r="A97" s="46">
         <v>95</v>
       </c>
@@ -13330,7 +13411,7 @@
       <c r="X97" s="48"/>
       <c r="Y97" s="67"/>
     </row>
-    <row r="98" ht="122.25" hidden="1" customHeight="1" spans="1:25">
+    <row r="98" ht="122.25" customHeight="1" spans="1:25">
       <c r="A98" s="46">
         <v>96</v>
       </c>
@@ -13359,7 +13440,7 @@
       <c r="X98" s="48"/>
       <c r="Y98" s="67"/>
     </row>
-    <row r="99" ht="16.5" hidden="1" spans="1:25">
+    <row r="99" ht="16.5" spans="1:25">
       <c r="A99" s="46">
         <v>97</v>
       </c>
@@ -13388,7 +13469,7 @@
       <c r="X99" s="48"/>
       <c r="Y99" s="67"/>
     </row>
-    <row r="100" ht="16.5" hidden="1" spans="1:25">
+    <row r="100" ht="16.5" spans="1:25">
       <c r="A100" s="46">
         <v>98</v>
       </c>
@@ -13417,7 +13498,7 @@
       <c r="X100" s="48"/>
       <c r="Y100" s="67"/>
     </row>
-    <row r="101" ht="16.5" hidden="1" spans="1:25">
+    <row r="101" ht="16.5" spans="1:25">
       <c r="A101" s="46">
         <v>99</v>
       </c>
@@ -13446,7 +13527,7 @@
       <c r="X101" s="48"/>
       <c r="Y101" s="67"/>
     </row>
-    <row r="102" ht="16.5" hidden="1" spans="1:25">
+    <row r="102" ht="16.5" spans="1:25">
       <c r="A102" s="46">
         <v>100</v>
       </c>
@@ -13475,7 +13556,7 @@
       <c r="X102" s="48"/>
       <c r="Y102" s="67"/>
     </row>
-    <row r="103" ht="16.5" hidden="1" spans="1:25">
+    <row r="103" ht="16.5" spans="1:25">
       <c r="A103" s="46">
         <v>101</v>
       </c>
@@ -13504,7 +13585,7 @@
       <c r="X103" s="48"/>
       <c r="Y103" s="67"/>
     </row>
-    <row r="104" ht="16.5" hidden="1" spans="1:25">
+    <row r="104" ht="16.5" spans="1:25">
       <c r="A104" s="46">
         <v>102</v>
       </c>
@@ -13533,7 +13614,7 @@
       <c r="X104" s="48"/>
       <c r="Y104" s="67"/>
     </row>
-    <row r="105" ht="16.5" hidden="1" spans="1:25">
+    <row r="105" ht="16.5" spans="1:25">
       <c r="A105" s="46">
         <v>103</v>
       </c>
@@ -13562,7 +13643,7 @@
       <c r="X105" s="48"/>
       <c r="Y105" s="67"/>
     </row>
-    <row r="106" ht="16.5" hidden="1" spans="1:25">
+    <row r="106" ht="16.5" spans="1:25">
       <c r="A106" s="46">
         <v>104</v>
       </c>
@@ -13591,12 +13672,12 @@
       <c r="X106" s="48"/>
       <c r="Y106" s="67"/>
     </row>
-    <row r="107" ht="16.5" hidden="1" spans="1:25">
+    <row r="107" ht="16.5" spans="1:25">
       <c r="A107" s="46">
         <v>105</v>
       </c>
       <c r="B107" s="48"/>
-      <c r="C107" s="112"/>
+      <c r="C107" s="111"/>
       <c r="D107" s="63"/>
       <c r="E107" s="69"/>
       <c r="F107" s="69"/>
@@ -13620,7 +13701,7 @@
       <c r="X107" s="48"/>
       <c r="Y107" s="67"/>
     </row>
-    <row r="108" ht="16.5" hidden="1" spans="1:25">
+    <row r="108" ht="16.5" spans="1:25">
       <c r="A108" s="46">
         <v>106</v>
       </c>
@@ -13649,7 +13730,7 @@
       <c r="X108" s="48"/>
       <c r="Y108" s="67"/>
     </row>
-    <row r="109" ht="16.5" hidden="1" spans="1:25">
+    <row r="109" ht="16.5" spans="1:25">
       <c r="A109" s="46">
         <v>107</v>
       </c>
@@ -13678,7 +13759,7 @@
       <c r="X109" s="48"/>
       <c r="Y109" s="67"/>
     </row>
-    <row r="110" ht="14.25" hidden="1" spans="1:25">
+    <row r="110" ht="14.25" spans="1:25">
       <c r="A110" s="46">
         <v>108</v>
       </c>
@@ -13707,7 +13788,7 @@
       <c r="X110" s="48"/>
       <c r="Y110" s="67"/>
     </row>
-    <row r="111" ht="16.5" hidden="1" spans="1:25">
+    <row r="111" ht="16.5" spans="1:25">
       <c r="A111" s="46">
         <v>109</v>
       </c>
@@ -13729,14 +13810,14 @@
       <c r="Q111" s="53"/>
       <c r="R111" s="53"/>
       <c r="S111" s="66"/>
-      <c r="T111" s="113"/>
+      <c r="T111" s="112"/>
       <c r="U111" s="48"/>
       <c r="V111" s="48"/>
       <c r="W111" s="48"/>
       <c r="X111" s="48"/>
       <c r="Y111" s="67"/>
     </row>
-    <row r="112" ht="16.5" hidden="1" spans="1:25">
+    <row r="112" ht="16.5" spans="1:25">
       <c r="A112" s="46">
         <v>110</v>
       </c>
@@ -13758,14 +13839,14 @@
       <c r="Q112" s="53"/>
       <c r="R112" s="53"/>
       <c r="S112" s="66"/>
-      <c r="T112" s="113"/>
+      <c r="T112" s="112"/>
       <c r="U112" s="48"/>
       <c r="V112" s="48"/>
       <c r="W112" s="48"/>
       <c r="X112" s="48"/>
       <c r="Y112" s="67"/>
     </row>
-    <row r="113" ht="16.5" hidden="1" spans="1:25">
+    <row r="113" ht="16.5" spans="1:25">
       <c r="A113" s="46">
         <v>111</v>
       </c>
@@ -13794,7 +13875,7 @@
       <c r="X113" s="48"/>
       <c r="Y113" s="67"/>
     </row>
-    <row r="114" ht="16.5" hidden="1" spans="1:25">
+    <row r="114" ht="16.5" spans="1:25">
       <c r="A114" s="46">
         <v>112</v>
       </c>
@@ -13816,14 +13897,14 @@
       <c r="Q114" s="53"/>
       <c r="R114" s="53"/>
       <c r="S114" s="66"/>
-      <c r="T114" s="113"/>
+      <c r="T114" s="112"/>
       <c r="U114" s="48"/>
       <c r="V114" s="48"/>
       <c r="W114" s="48"/>
       <c r="X114" s="48"/>
       <c r="Y114" s="67"/>
     </row>
-    <row r="115" ht="16.5" hidden="1" spans="1:25">
+    <row r="115" ht="16.5" spans="1:25">
       <c r="A115" s="46">
         <v>113</v>
       </c>
@@ -13851,7 +13932,7 @@
       <c r="W115" s="48"/>
       <c r="X115" s="48"/>
     </row>
-    <row r="116" ht="16.5" hidden="1" spans="1:25">
+    <row r="116" ht="16.5" spans="1:25">
       <c r="A116" s="46">
         <v>114</v>
       </c>
@@ -13873,13 +13954,13 @@
       <c r="Q116" s="53"/>
       <c r="R116" s="53"/>
       <c r="S116" s="66"/>
-      <c r="T116" s="113"/>
+      <c r="T116" s="112"/>
       <c r="U116" s="48"/>
       <c r="V116" s="48"/>
       <c r="W116" s="48"/>
       <c r="X116" s="48"/>
     </row>
-    <row r="117" hidden="1" customHeight="1" spans="1:25">
+    <row r="117" customHeight="1" spans="1:25">
       <c r="A117" s="46">
         <v>115</v>
       </c>
@@ -13907,7 +13988,7 @@
       <c r="W117" s="48"/>
       <c r="X117" s="48"/>
     </row>
-    <row r="118" hidden="1" customHeight="1" spans="1:25">
+    <row r="118" customHeight="1" spans="1:25">
       <c r="A118" s="46">
         <v>116</v>
       </c>
@@ -13935,35 +14016,35 @@
       <c r="W118" s="48"/>
       <c r="X118" s="48"/>
     </row>
-    <row r="119" hidden="1" customHeight="1" spans="1:25">
+    <row r="119" customHeight="1" spans="1:25">
       <c r="A119" s="46">
         <v>117</v>
       </c>
-      <c r="B119" s="114"/>
-      <c r="C119" s="114"/>
-      <c r="D119" s="115"/>
-      <c r="E119" s="116"/>
-      <c r="F119" s="116"/>
-      <c r="G119" s="116"/>
-      <c r="H119" s="116"/>
-      <c r="I119" s="115"/>
-      <c r="J119" s="114"/>
-      <c r="K119" s="117"/>
-      <c r="L119" s="118"/>
-      <c r="M119" s="118"/>
-      <c r="N119" s="114"/>
-      <c r="O119" s="114"/>
-      <c r="P119" s="114"/>
-      <c r="Q119" s="118"/>
-      <c r="R119" s="118"/>
-      <c r="S119" s="119"/>
-      <c r="T119" s="114"/>
-      <c r="U119" s="114"/>
-      <c r="V119" s="114"/>
-      <c r="W119" s="114"/>
-      <c r="X119" s="114"/>
-    </row>
-    <row r="120" ht="135" hidden="1" customHeight="1" spans="1:25">
+      <c r="B119" s="113"/>
+      <c r="C119" s="113"/>
+      <c r="D119" s="114"/>
+      <c r="E119" s="115"/>
+      <c r="F119" s="115"/>
+      <c r="G119" s="115"/>
+      <c r="H119" s="115"/>
+      <c r="I119" s="114"/>
+      <c r="J119" s="113"/>
+      <c r="K119" s="116"/>
+      <c r="L119" s="117"/>
+      <c r="M119" s="117"/>
+      <c r="N119" s="113"/>
+      <c r="O119" s="113"/>
+      <c r="P119" s="113"/>
+      <c r="Q119" s="117"/>
+      <c r="R119" s="117"/>
+      <c r="S119" s="118"/>
+      <c r="T119" s="113"/>
+      <c r="U119" s="113"/>
+      <c r="V119" s="113"/>
+      <c r="W119" s="113"/>
+      <c r="X119" s="113"/>
+    </row>
+    <row r="120" ht="135" customHeight="1" spans="1:25">
       <c r="A120" s="46">
         <v>118</v>
       </c>
@@ -13992,7 +14073,7 @@
       <c r="X120" s="48"/>
       <c r="Y120" s="67"/>
     </row>
-    <row r="121" ht="108" hidden="1" customHeight="1" spans="1:25">
+    <row r="121" ht="108" customHeight="1" spans="1:25">
       <c r="A121" s="46">
         <v>119</v>
       </c>
@@ -14016,26 +14097,26 @@
       <c r="S121" s="66"/>
       <c r="T121" s="48"/>
       <c r="U121" s="48"/>
-      <c r="V121" s="114"/>
-      <c r="W121" s="114"/>
+      <c r="V121" s="113"/>
+      <c r="W121" s="113"/>
       <c r="X121" s="48"/>
       <c r="Y121" s="67"/>
     </row>
-    <row r="122" ht="187.5" hidden="1" customHeight="1" spans="1:25">
+    <row r="122" ht="187.5" customHeight="1" spans="1:25">
       <c r="A122" s="46">
         <v>120</v>
       </c>
       <c r="B122" s="48"/>
       <c r="C122" s="48"/>
       <c r="D122" s="63"/>
-      <c r="E122" s="120"/>
-      <c r="F122" s="120"/>
-      <c r="G122" s="120"/>
-      <c r="H122" s="120"/>
+      <c r="E122" s="119"/>
+      <c r="F122" s="119"/>
+      <c r="G122" s="119"/>
+      <c r="H122" s="119"/>
       <c r="I122" s="63"/>
       <c r="J122" s="48"/>
       <c r="K122" s="65"/>
-      <c r="L122" s="121"/>
+      <c r="L122" s="120"/>
       <c r="M122" s="53"/>
       <c r="N122" s="48"/>
       <c r="O122" s="48"/>
@@ -14050,17 +14131,17 @@
       <c r="X122" s="48"/>
       <c r="Y122" s="53"/>
     </row>
-    <row r="123" hidden="1" customHeight="1" spans="1:25">
+    <row r="123" customHeight="1" spans="1:25">
       <c r="A123" s="46">
         <v>121</v>
       </c>
       <c r="B123" s="48"/>
       <c r="C123" s="48"/>
       <c r="D123" s="63"/>
-      <c r="E123" s="120"/>
-      <c r="F123" s="120"/>
-      <c r="G123" s="120"/>
-      <c r="H123" s="120"/>
+      <c r="E123" s="119"/>
+      <c r="F123" s="119"/>
+      <c r="G123" s="119"/>
+      <c r="H123" s="119"/>
       <c r="I123" s="63"/>
       <c r="J123" s="48"/>
       <c r="K123" s="65"/>
@@ -14079,17 +14160,17 @@
       <c r="X123" s="48"/>
       <c r="Y123" s="67"/>
     </row>
-    <row r="124" ht="141.6" hidden="1" customHeight="1" spans="1:25">
+    <row r="124" ht="141.6" customHeight="1" spans="1:25">
       <c r="A124" s="46">
         <v>122</v>
       </c>
       <c r="B124" s="48"/>
       <c r="C124" s="48"/>
       <c r="D124" s="63"/>
-      <c r="E124" s="120"/>
-      <c r="F124" s="120"/>
-      <c r="G124" s="120"/>
-      <c r="H124" s="120"/>
+      <c r="E124" s="119"/>
+      <c r="F124" s="119"/>
+      <c r="G124" s="119"/>
+      <c r="H124" s="119"/>
       <c r="I124" s="63"/>
       <c r="J124" s="48"/>
       <c r="K124" s="65"/>
@@ -14108,17 +14189,17 @@
       <c r="X124" s="48"/>
       <c r="Y124" s="67"/>
     </row>
-    <row r="125" ht="16.5" hidden="1" spans="1:25">
+    <row r="125" ht="16.5" spans="1:25">
       <c r="A125" s="46">
         <v>123</v>
       </c>
       <c r="B125" s="48"/>
       <c r="C125" s="48"/>
       <c r="D125" s="63"/>
-      <c r="E125" s="120"/>
-      <c r="F125" s="120"/>
-      <c r="G125" s="120"/>
-      <c r="H125" s="120"/>
+      <c r="E125" s="119"/>
+      <c r="F125" s="119"/>
+      <c r="G125" s="119"/>
+      <c r="H125" s="119"/>
       <c r="I125" s="63"/>
       <c r="J125" s="48"/>
       <c r="K125" s="65"/>
@@ -14137,17 +14218,17 @@
       <c r="X125" s="48"/>
       <c r="Y125" s="67"/>
     </row>
-    <row r="126" ht="16.5" hidden="1" spans="1:25">
+    <row r="126" ht="16.5" spans="1:25">
       <c r="A126" s="46">
         <v>124</v>
       </c>
       <c r="B126" s="48"/>
       <c r="C126" s="48"/>
       <c r="D126" s="63"/>
-      <c r="E126" s="120"/>
-      <c r="F126" s="120"/>
-      <c r="G126" s="120"/>
-      <c r="H126" s="120"/>
+      <c r="E126" s="119"/>
+      <c r="F126" s="119"/>
+      <c r="G126" s="119"/>
+      <c r="H126" s="119"/>
       <c r="I126" s="63"/>
       <c r="J126" s="48"/>
       <c r="K126" s="65"/>
@@ -14166,17 +14247,17 @@
       <c r="X126" s="48"/>
       <c r="Y126" s="67"/>
     </row>
-    <row r="127" ht="316.15" hidden="1" customHeight="1" spans="1:25">
+    <row r="127" ht="316.15" customHeight="1" spans="1:25">
       <c r="A127" s="46">
         <v>125</v>
       </c>
       <c r="B127" s="48"/>
       <c r="C127" s="48"/>
       <c r="D127" s="63"/>
-      <c r="E127" s="120"/>
-      <c r="F127" s="120"/>
-      <c r="G127" s="120"/>
-      <c r="H127" s="120"/>
+      <c r="E127" s="119"/>
+      <c r="F127" s="119"/>
+      <c r="G127" s="119"/>
+      <c r="H127" s="119"/>
       <c r="I127" s="63"/>
       <c r="J127" s="48"/>
       <c r="K127" s="65"/>
@@ -14195,7 +14276,7 @@
       <c r="X127" s="48"/>
       <c r="Y127" s="67"/>
     </row>
-    <row r="128" ht="165.75" hidden="1" customHeight="1" spans="1:25">
+    <row r="128" ht="165.75" customHeight="1" spans="1:25">
       <c r="A128" s="46">
         <v>126</v>
       </c>
@@ -14215,8 +14296,8 @@
       <c r="O128" s="48"/>
       <c r="P128" s="48"/>
       <c r="Q128" s="53"/>
-      <c r="R128" s="113"/>
-      <c r="S128" s="113"/>
+      <c r="R128" s="112"/>
+      <c r="S128" s="112"/>
       <c r="T128" s="48"/>
       <c r="U128" s="48"/>
       <c r="V128" s="48"/>
@@ -14224,7 +14305,7 @@
       <c r="X128" s="48"/>
       <c r="Y128" s="67"/>
     </row>
-    <row r="129" ht="16.5" hidden="1" spans="1:25">
+    <row r="129" ht="16.5" spans="1:25">
       <c r="A129" s="46">
         <v>127</v>
       </c>
@@ -14244,8 +14325,8 @@
       <c r="O129" s="48"/>
       <c r="P129" s="48"/>
       <c r="Q129" s="53"/>
-      <c r="R129" s="122"/>
-      <c r="S129" s="123"/>
+      <c r="R129" s="121"/>
+      <c r="S129" s="122"/>
       <c r="T129" s="48"/>
       <c r="U129" s="48"/>
       <c r="V129" s="48"/>
@@ -14253,7 +14334,7 @@
       <c r="X129" s="48"/>
       <c r="Y129" s="67"/>
     </row>
-    <row r="130" ht="16.5" hidden="1" spans="1:25">
+    <row r="130" ht="16.5" spans="1:25">
       <c r="A130" s="46">
         <v>128</v>
       </c>
@@ -14282,7 +14363,7 @@
       <c r="X130" s="48"/>
       <c r="Y130" s="67"/>
     </row>
-    <row r="131" ht="16.5" hidden="1" spans="1:25">
+    <row r="131" ht="16.5" spans="1:25">
       <c r="A131" s="46">
         <v>129</v>
       </c>
@@ -14311,7 +14392,7 @@
       <c r="X131" s="48"/>
       <c r="Y131" s="67"/>
     </row>
-    <row r="132" ht="16.5" hidden="1" spans="1:25">
+    <row r="132" ht="16.5" spans="1:25">
       <c r="A132" s="46">
         <v>130</v>
       </c>
@@ -14340,7 +14421,7 @@
       <c r="X132" s="48"/>
       <c r="Y132" s="67"/>
     </row>
-    <row r="133" ht="181.5" hidden="1" customHeight="1" spans="1:25">
+    <row r="133" ht="181.5" customHeight="1" spans="1:25">
       <c r="A133" s="46">
         <v>131</v>
       </c>
@@ -14369,7 +14450,7 @@
       <c r="X133" s="48"/>
       <c r="Y133" s="67"/>
     </row>
-    <row r="134" ht="150.75" hidden="1" customHeight="1" spans="1:25">
+    <row r="134" ht="150.75" customHeight="1" spans="1:25">
       <c r="A134" s="46">
         <v>132</v>
       </c>
@@ -14398,17 +14479,17 @@
       <c r="X134" s="48"/>
       <c r="Y134" s="67"/>
     </row>
-    <row r="135" ht="108" hidden="1" customHeight="1" spans="1:25">
+    <row r="135" ht="108" customHeight="1" spans="1:25">
       <c r="A135" s="46">
         <v>133</v>
       </c>
       <c r="B135" s="48"/>
       <c r="C135" s="48"/>
       <c r="D135" s="63"/>
-      <c r="E135" s="120"/>
-      <c r="F135" s="120"/>
-      <c r="G135" s="120"/>
-      <c r="H135" s="120"/>
+      <c r="E135" s="119"/>
+      <c r="F135" s="119"/>
+      <c r="G135" s="119"/>
+      <c r="H135" s="119"/>
       <c r="I135" s="63"/>
       <c r="J135" s="48"/>
       <c r="K135" s="65"/>
@@ -14427,17 +14508,17 @@
       <c r="X135" s="48"/>
       <c r="Y135" s="67"/>
     </row>
-    <row r="136" ht="16.5" hidden="1" spans="1:25">
+    <row r="136" ht="16.5" spans="1:25">
       <c r="A136" s="46">
         <v>134</v>
       </c>
       <c r="B136" s="48"/>
       <c r="C136" s="48"/>
       <c r="D136" s="63"/>
-      <c r="E136" s="120"/>
-      <c r="F136" s="120"/>
-      <c r="G136" s="120"/>
-      <c r="H136" s="120"/>
+      <c r="E136" s="119"/>
+      <c r="F136" s="119"/>
+      <c r="G136" s="119"/>
+      <c r="H136" s="119"/>
       <c r="I136" s="63"/>
       <c r="J136" s="48"/>
       <c r="K136" s="65"/>
@@ -14456,17 +14537,17 @@
       <c r="X136" s="48"/>
       <c r="Y136" s="67"/>
     </row>
-    <row r="137" ht="16.5" hidden="1" spans="1:25">
+    <row r="137" ht="16.5" spans="1:25">
       <c r="A137" s="46">
         <v>135</v>
       </c>
       <c r="B137" s="48"/>
       <c r="C137" s="48"/>
       <c r="D137" s="63"/>
-      <c r="E137" s="120"/>
-      <c r="F137" s="120"/>
-      <c r="G137" s="120"/>
-      <c r="H137" s="120"/>
+      <c r="E137" s="119"/>
+      <c r="F137" s="119"/>
+      <c r="G137" s="119"/>
+      <c r="H137" s="119"/>
       <c r="I137" s="63"/>
       <c r="J137" s="48"/>
       <c r="K137" s="65"/>
@@ -14485,7 +14566,7 @@
       <c r="X137" s="48"/>
       <c r="Y137" s="67"/>
     </row>
-    <row r="138" ht="16.5" hidden="1" spans="1:25">
+    <row r="138" ht="16.5" spans="1:25">
       <c r="A138" s="46">
         <v>136</v>
       </c>
@@ -14495,7 +14576,7 @@
       <c r="E138" s="69"/>
       <c r="F138" s="69"/>
       <c r="G138" s="69"/>
-      <c r="H138" s="120"/>
+      <c r="H138" s="119"/>
       <c r="I138" s="63"/>
       <c r="J138" s="48"/>
       <c r="K138" s="65"/>
@@ -14514,17 +14595,17 @@
       <c r="X138" s="48"/>
       <c r="Y138" s="67"/>
     </row>
-    <row r="139" ht="16.5" hidden="1" spans="1:25">
+    <row r="139" ht="16.5" spans="1:25">
       <c r="A139" s="46">
         <v>137</v>
       </c>
       <c r="B139" s="48"/>
       <c r="C139" s="48"/>
       <c r="D139" s="63"/>
-      <c r="E139" s="120"/>
-      <c r="F139" s="120"/>
-      <c r="G139" s="120"/>
-      <c r="H139" s="120"/>
+      <c r="E139" s="119"/>
+      <c r="F139" s="119"/>
+      <c r="G139" s="119"/>
+      <c r="H139" s="119"/>
       <c r="I139" s="63"/>
       <c r="J139" s="48"/>
       <c r="K139" s="65"/>
@@ -14543,17 +14624,17 @@
       <c r="X139" s="48"/>
       <c r="Y139" s="67"/>
     </row>
-    <row r="140" ht="16.5" hidden="1" spans="1:25">
+    <row r="140" ht="16.5" spans="1:25">
       <c r="A140" s="46">
         <v>138</v>
       </c>
       <c r="B140" s="48"/>
       <c r="C140" s="48"/>
       <c r="D140" s="63"/>
-      <c r="E140" s="124"/>
-      <c r="F140" s="120"/>
-      <c r="G140" s="120"/>
-      <c r="H140" s="120"/>
+      <c r="E140" s="123"/>
+      <c r="F140" s="119"/>
+      <c r="G140" s="119"/>
+      <c r="H140" s="119"/>
       <c r="I140" s="63"/>
       <c r="J140" s="48"/>
       <c r="K140" s="65"/>
@@ -14572,17 +14653,17 @@
       <c r="X140" s="48"/>
       <c r="Y140" s="67"/>
     </row>
-    <row r="141" ht="16.5" hidden="1" spans="1:25">
+    <row r="141" ht="16.5" spans="1:25">
       <c r="A141" s="46">
         <v>139</v>
       </c>
       <c r="B141" s="48"/>
       <c r="C141" s="48"/>
       <c r="D141" s="63"/>
-      <c r="E141" s="120"/>
-      <c r="F141" s="120"/>
-      <c r="G141" s="120"/>
-      <c r="H141" s="120"/>
+      <c r="E141" s="119"/>
+      <c r="F141" s="119"/>
+      <c r="G141" s="119"/>
+      <c r="H141" s="119"/>
       <c r="I141" s="63"/>
       <c r="J141" s="48"/>
       <c r="K141" s="65"/>
@@ -14601,17 +14682,17 @@
       <c r="X141" s="48"/>
       <c r="Y141" s="67"/>
     </row>
-    <row r="142" ht="16.5" hidden="1" spans="1:25">
+    <row r="142" ht="16.5" spans="1:25">
       <c r="A142" s="46">
         <v>140</v>
       </c>
       <c r="B142" s="48"/>
       <c r="C142" s="48"/>
       <c r="D142" s="63"/>
-      <c r="E142" s="120"/>
-      <c r="F142" s="120"/>
-      <c r="G142" s="120"/>
-      <c r="H142" s="120"/>
+      <c r="E142" s="119"/>
+      <c r="F142" s="119"/>
+      <c r="G142" s="119"/>
+      <c r="H142" s="119"/>
       <c r="I142" s="63"/>
       <c r="J142" s="48"/>
       <c r="K142" s="65"/>
@@ -14630,17 +14711,17 @@
       <c r="X142" s="48"/>
       <c r="Y142" s="67"/>
     </row>
-    <row r="143" ht="16.5" hidden="1" spans="1:25">
+    <row r="143" ht="16.5" spans="1:25">
       <c r="A143" s="46">
         <v>141</v>
       </c>
       <c r="B143" s="48"/>
       <c r="C143" s="48"/>
       <c r="D143" s="63"/>
-      <c r="E143" s="120"/>
-      <c r="F143" s="120"/>
-      <c r="G143" s="120"/>
-      <c r="H143" s="120"/>
+      <c r="E143" s="119"/>
+      <c r="F143" s="119"/>
+      <c r="G143" s="119"/>
+      <c r="H143" s="119"/>
       <c r="I143" s="63"/>
       <c r="J143" s="48"/>
       <c r="K143" s="65"/>
@@ -14659,14 +14740,14 @@
       <c r="X143" s="48"/>
       <c r="Y143" s="67"/>
     </row>
-    <row r="144" ht="16.5" hidden="1" spans="1:25">
+    <row r="144" ht="16.5" spans="1:25">
       <c r="A144" s="46">
         <v>142</v>
       </c>
       <c r="B144" s="48"/>
       <c r="C144" s="48"/>
       <c r="D144" s="63"/>
-      <c r="E144" s="124"/>
+      <c r="E144" s="123"/>
       <c r="F144" s="50"/>
       <c r="G144" s="50"/>
       <c r="H144" s="50"/>
@@ -14680,7 +14761,7 @@
       <c r="P144" s="48"/>
       <c r="Q144" s="53"/>
       <c r="R144" s="53"/>
-      <c r="S144" s="123"/>
+      <c r="S144" s="122"/>
       <c r="T144" s="48"/>
       <c r="U144" s="48"/>
       <c r="V144" s="48"/>
@@ -14688,7 +14769,7 @@
       <c r="X144" s="48"/>
       <c r="Y144" s="67"/>
     </row>
-    <row r="145" ht="16.5" hidden="1" spans="1:25">
+    <row r="145" ht="16.5" spans="1:25">
       <c r="A145" s="46">
         <v>143</v>
       </c>
@@ -14717,7 +14798,7 @@
       <c r="X145" s="48"/>
       <c r="Y145" s="67"/>
     </row>
-    <row r="146" ht="16.5" hidden="1" spans="1:25">
+    <row r="146" ht="16.5" spans="1:25">
       <c r="A146" s="46">
         <v>144</v>
       </c>
@@ -14746,7 +14827,7 @@
       <c r="X146" s="48"/>
       <c r="Y146" s="67"/>
     </row>
-    <row r="147" ht="16.5" hidden="1" spans="1:25">
+    <row r="147" ht="16.5" spans="1:25">
       <c r="A147" s="46">
         <v>145</v>
       </c>
@@ -14756,7 +14837,7 @@
       <c r="E147" s="64"/>
       <c r="F147" s="64"/>
       <c r="G147" s="64"/>
-      <c r="H147" s="120"/>
+      <c r="H147" s="119"/>
       <c r="I147" s="63"/>
       <c r="J147" s="48"/>
       <c r="K147" s="65"/>
@@ -14775,7 +14856,7 @@
       <c r="X147" s="48"/>
       <c r="Y147" s="67"/>
     </row>
-    <row r="148" ht="16.5" hidden="1" spans="1:25">
+    <row r="148" ht="16.5" spans="1:25">
       <c r="A148" s="46">
         <v>146</v>
       </c>
@@ -14785,7 +14866,7 @@
       <c r="E148" s="64"/>
       <c r="F148" s="64"/>
       <c r="G148" s="64"/>
-      <c r="H148" s="120"/>
+      <c r="H148" s="119"/>
       <c r="I148" s="63"/>
       <c r="J148" s="48"/>
       <c r="K148" s="65"/>
@@ -14804,7 +14885,7 @@
       <c r="X148" s="48"/>
       <c r="Y148" s="67"/>
     </row>
-    <row r="149" ht="16.5" hidden="1" spans="1:25">
+    <row r="149" ht="16.5" spans="1:25">
       <c r="A149" s="46">
         <v>147</v>
       </c>
@@ -14833,7 +14914,7 @@
       <c r="X149" s="48"/>
       <c r="Y149" s="67"/>
     </row>
-    <row r="150" ht="16.5" hidden="1" spans="1:25">
+    <row r="150" ht="16.5" spans="1:25">
       <c r="A150" s="46">
         <v>148</v>
       </c>
@@ -14843,7 +14924,7 @@
       <c r="E150" s="64"/>
       <c r="F150" s="64"/>
       <c r="G150" s="64"/>
-      <c r="H150" s="120"/>
+      <c r="H150" s="119"/>
       <c r="I150" s="63"/>
       <c r="J150" s="48"/>
       <c r="K150" s="65"/>
@@ -14862,7 +14943,7 @@
       <c r="X150" s="48"/>
       <c r="Y150" s="67"/>
     </row>
-    <row r="151" ht="16.5" hidden="1" spans="1:25">
+    <row r="151" ht="16.5" spans="1:25">
       <c r="A151" s="46">
         <v>149</v>
       </c>
@@ -14891,7 +14972,7 @@
       <c r="X151" s="48"/>
       <c r="Y151" s="67"/>
     </row>
-    <row r="152" ht="16.5" hidden="1" spans="1:25">
+    <row r="152" ht="16.5" spans="1:25">
       <c r="A152" s="46">
         <v>150</v>
       </c>
@@ -14920,17 +15001,17 @@
       <c r="X152" s="48"/>
       <c r="Y152" s="67"/>
     </row>
-    <row r="153" hidden="1" customHeight="1" spans="1:25">
+    <row r="153" customHeight="1" spans="1:25">
       <c r="A153" s="46">
         <v>151</v>
       </c>
       <c r="B153" s="48"/>
       <c r="C153" s="48"/>
       <c r="D153" s="63"/>
-      <c r="E153" s="120"/>
-      <c r="F153" s="120"/>
-      <c r="G153" s="120"/>
-      <c r="H153" s="120"/>
+      <c r="E153" s="119"/>
+      <c r="F153" s="119"/>
+      <c r="G153" s="119"/>
+      <c r="H153" s="119"/>
       <c r="I153" s="63"/>
       <c r="J153" s="48"/>
       <c r="K153" s="65"/>
@@ -14949,17 +15030,17 @@
       <c r="X153" s="48"/>
       <c r="Y153" s="67"/>
     </row>
-    <row r="154" hidden="1" customHeight="1" spans="1:25">
+    <row r="154" customHeight="1" spans="1:25">
       <c r="A154" s="46">
         <v>152</v>
       </c>
       <c r="B154" s="48"/>
       <c r="C154" s="48"/>
       <c r="D154" s="63"/>
-      <c r="E154" s="120"/>
-      <c r="F154" s="120"/>
-      <c r="G154" s="120"/>
-      <c r="H154" s="120"/>
+      <c r="E154" s="119"/>
+      <c r="F154" s="119"/>
+      <c r="G154" s="119"/>
+      <c r="H154" s="119"/>
       <c r="I154" s="63"/>
       <c r="J154" s="48"/>
       <c r="K154" s="65"/>
@@ -14978,17 +15059,17 @@
       <c r="X154" s="48"/>
       <c r="Y154" s="67"/>
     </row>
-    <row r="155" hidden="1" customHeight="1" spans="1:25">
+    <row r="155" customHeight="1" spans="1:25">
       <c r="A155" s="46">
         <v>153</v>
       </c>
       <c r="B155" s="48"/>
       <c r="C155" s="48"/>
       <c r="D155" s="63"/>
-      <c r="E155" s="120"/>
-      <c r="F155" s="120"/>
-      <c r="G155" s="120"/>
-      <c r="H155" s="120"/>
+      <c r="E155" s="119"/>
+      <c r="F155" s="119"/>
+      <c r="G155" s="119"/>
+      <c r="H155" s="119"/>
       <c r="I155" s="63"/>
       <c r="J155" s="48"/>
       <c r="K155" s="65"/>
@@ -15007,17 +15088,17 @@
       <c r="X155" s="48"/>
       <c r="Y155" s="67"/>
     </row>
-    <row r="156" hidden="1" customHeight="1" spans="1:25">
+    <row r="156" customHeight="1" spans="1:25">
       <c r="A156" s="46">
         <v>154</v>
       </c>
       <c r="B156" s="48"/>
       <c r="C156" s="48"/>
       <c r="D156" s="63"/>
-      <c r="E156" s="120"/>
-      <c r="F156" s="120"/>
-      <c r="G156" s="120"/>
-      <c r="H156" s="120"/>
+      <c r="E156" s="119"/>
+      <c r="F156" s="119"/>
+      <c r="G156" s="119"/>
+      <c r="H156" s="119"/>
       <c r="I156" s="63"/>
       <c r="J156" s="48"/>
       <c r="K156" s="65"/>
@@ -15036,17 +15117,17 @@
       <c r="X156" s="48"/>
       <c r="Y156" s="67"/>
     </row>
-    <row r="157" hidden="1" customHeight="1" spans="1:25">
+    <row r="157" customHeight="1" spans="1:25">
       <c r="A157" s="46">
         <v>155</v>
       </c>
       <c r="B157" s="48"/>
       <c r="C157" s="48"/>
       <c r="D157" s="63"/>
-      <c r="E157" s="120"/>
-      <c r="F157" s="120"/>
-      <c r="G157" s="120"/>
-      <c r="H157" s="120"/>
+      <c r="E157" s="119"/>
+      <c r="F157" s="119"/>
+      <c r="G157" s="119"/>
+      <c r="H157" s="119"/>
       <c r="I157" s="63"/>
       <c r="J157" s="48"/>
       <c r="K157" s="65"/>
@@ -15065,17 +15146,17 @@
       <c r="X157" s="48"/>
       <c r="Y157" s="67"/>
     </row>
-    <row r="158" hidden="1" customHeight="1" spans="1:25">
+    <row r="158" customHeight="1" spans="1:25">
       <c r="A158" s="46">
         <v>156</v>
       </c>
       <c r="B158" s="48"/>
       <c r="C158" s="48"/>
       <c r="D158" s="63"/>
-      <c r="E158" s="120"/>
-      <c r="F158" s="120"/>
-      <c r="G158" s="120"/>
-      <c r="H158" s="120"/>
+      <c r="E158" s="119"/>
+      <c r="F158" s="119"/>
+      <c r="G158" s="119"/>
+      <c r="H158" s="119"/>
       <c r="I158" s="63"/>
       <c r="J158" s="48"/>
       <c r="K158" s="65"/>
@@ -15094,17 +15175,17 @@
       <c r="X158" s="48"/>
       <c r="Y158" s="67"/>
     </row>
-    <row r="159" hidden="1" customHeight="1" spans="1:25">
+    <row r="159" customHeight="1" spans="1:25">
       <c r="A159" s="46">
         <v>157</v>
       </c>
       <c r="B159" s="48"/>
       <c r="C159" s="48"/>
       <c r="D159" s="63"/>
-      <c r="E159" s="120"/>
-      <c r="F159" s="120"/>
-      <c r="G159" s="120"/>
-      <c r="H159" s="120"/>
+      <c r="E159" s="119"/>
+      <c r="F159" s="119"/>
+      <c r="G159" s="119"/>
+      <c r="H159" s="119"/>
       <c r="I159" s="63"/>
       <c r="J159" s="48"/>
       <c r="K159" s="65"/>
@@ -15123,17 +15204,17 @@
       <c r="X159" s="48"/>
       <c r="Y159" s="67"/>
     </row>
-    <row r="160" hidden="1" customHeight="1" spans="1:25">
+    <row r="160" customHeight="1" spans="1:25">
       <c r="A160" s="46">
         <v>158</v>
       </c>
       <c r="B160" s="48"/>
       <c r="C160" s="48"/>
       <c r="D160" s="63"/>
-      <c r="E160" s="120"/>
-      <c r="F160" s="120"/>
-      <c r="G160" s="120"/>
-      <c r="H160" s="120"/>
+      <c r="E160" s="119"/>
+      <c r="F160" s="119"/>
+      <c r="G160" s="119"/>
+      <c r="H160" s="119"/>
       <c r="I160" s="63"/>
       <c r="J160" s="48"/>
       <c r="K160" s="65"/>
@@ -15152,16 +15233,10 @@
       <c r="X160" s="48"/>
       <c r="Y160" s="67"/>
     </row>
-    <row r="161" ht="13.5" hidden="1"/>
+    <row r="161" ht="13.5"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" insertColumns="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A2:Y161" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="15">
-      <customFilters>
-        <customFilter operator="equal" val="未结案"/>
-        <customFilter operator="equal" val="暂停"/>
-      </customFilters>
-    </filterColumn>
     <extLst/>
   </autoFilter>
   <mergeCells count="1">
@@ -15398,7 +15473,7 @@
   <sheetData>
     <row r="1" customHeight="1" spans="1:17">
       <c r="A1" s="8" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -15419,52 +15494,52 @@
     </row>
     <row r="2" s="1" customFormat="1" customHeight="1" spans="1:17">
       <c r="A2" s="9" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="L2" s="11" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="N2" s="9" t="s">
         <v>14</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="P2" s="13" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="Q2" s="9" t="s">
         <v>25</v>

</xml_diff>